<commit_message>
Taxonomy: preserve set size (3lü/4lü) in GenelUrunAdi for SET/SETİ products
</commit_message>
<xml_diff>
--- a/STOK_TAKSONOMT_DUZENLE.xlsx
+++ b/STOK_TAKSONOMT_DUZENLE.xlsx
@@ -1556,7 +1556,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>PLS. 4 LÜ DIAMOND YEMEK SETİ ŞEFFAF</t>
+          <t>PLS. DIAMOND YEMEK SETİ 4'lü ŞEFFAF</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>PLS. 4 LÜ PREMİUM YEMEK SETİ ŞEFFAF</t>
+          <t>PLS. PREMİUM YEMEK SETİ 4'lü ŞEFFAF</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>PLS. 3 LÜ DIAMOND YEMEK SETİ</t>
+          <t>PLS. DIAMOND YEMEK SETİ 3'lü</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>PLS. 4 LÜ DIAMOND YEMEK SETİ BEYAZ</t>
+          <t>PLS. DIAMOND YEMEK SETİ 4'lü BEYAZ</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
@@ -3647,7 +3647,7 @@
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>PLS. 3 LÜ DIAMOND YEMEK SETİ SİYAH</t>
+          <t>PLS. DIAMOND YEMEK SETİ 3'lü SİYAH</t>
         </is>
       </c>
       <c r="D77" s="8" t="inlineStr">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMİUM SET SİYAH</t>
+          <t>PLS. PREMİUM SET 4'lü SİYAH</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
@@ -3729,7 +3729,7 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>PLS. 6 LI PREMIUM YEMEK SETİ</t>
+          <t>PLS. PREMIUM YEMEK SETİ 6'lü</t>
         </is>
       </c>
       <c r="D79" s="8" t="inlineStr">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>PLS. 4 LÜ PREMIUM YEMEK SETİ BEYAZ</t>
+          <t>PLS. PREMIUM YEMEK SETİ 4'lü BEYAZ</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>FERPROM PLS. PREMIUM SET (ÇATAL+ BIÇAK)</t>
+          <t>FERPROM PLS. PREMIUM SET 3'lü (ÇATAL+ BIÇAK)</t>
         </is>
       </c>
       <c r="D87" s="8" t="inlineStr">
@@ -4098,7 +4098,7 @@
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>BEST PLS. YEMEK SET ŞEFFAF</t>
+          <t>BEST PLS. YEMEK SET 3'lü ŞEFFAF</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>PLS. ELİTE 4 LÜ YEMEK SETİ BEYAZ</t>
+          <t>PLS. ELİTE YEMEK SETİ 4'lü BEYAZ</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>PLS. ELİTE 3 LÜ YEMEK SETİ BEYAZ</t>
+          <t>PLS. ELİTE YEMEK SETİ 3'lü BEYAZ</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
@@ -4836,7 +4836,7 @@
       </c>
       <c r="C106" s="6" t="inlineStr">
         <is>
-          <t>PLS. 4 LÜ EKO YEMEK SETİ BEYAZ</t>
+          <t>PLS. EKO YEMEK SETİ 4'lü BEYAZ</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
@@ -5000,7 +5000,7 @@
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>BEST PLS. YEMEK SETi ŞEFFAF</t>
+          <t>BEST PLS. YEMEK SETi 4'lü ŞEFFAF</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="C113" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMIUM SET SİYAH</t>
+          <t>PLS. PREMIUM SET 3'lü SİYAH</t>
         </is>
       </c>
       <c r="D113" s="8" t="inlineStr">
@@ -5615,7 +5615,7 @@
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>PLS. 3 LÜ PREMIUM YEMEK SETİ BEYAZ</t>
+          <t>PLS. PREMIUM YEMEK SETİ 3'lü BEYAZ</t>
         </is>
       </c>
       <c r="D125" s="8" t="inlineStr">
@@ -5656,7 +5656,7 @@
       </c>
       <c r="C126" s="6" t="inlineStr">
         <is>
-          <t>PLS. 3 LÜ DIAMOND YEMEK SETİ BEYAZ</t>
+          <t>PLS. DIAMOND YEMEK SETİ 3'lü BEYAZ</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
@@ -6271,7 +6271,7 @@
       </c>
       <c r="C141" s="6" t="inlineStr">
         <is>
-          <t>6 LI SET SMARTPACK ŞEFFAF Ç+K</t>
+          <t>SET 6'lü SMARTPACK ŞEFFAF Ç+K</t>
         </is>
       </c>
       <c r="D141" s="8" t="inlineStr">
@@ -6476,7 +6476,7 @@
       </c>
       <c r="C146" s="6" t="inlineStr">
         <is>
-          <t>3'LÜ PREMİUM SET ÇATAL BIÇAK PEÇETE</t>
+          <t>PREMİUM SET 3'lü ÇATAL BIÇAK PEÇETE</t>
         </is>
       </c>
       <c r="D146" s="7" t="inlineStr">
@@ -7378,7 +7378,7 @@
       </c>
       <c r="C168" s="6" t="inlineStr">
         <is>
-          <t>PLS. 3 LÜ PREMIUM YEMEK SETİ BEYAZ</t>
+          <t>PLS. PREMIUM YEMEK SETİ 3'lü BEYAZ</t>
         </is>
       </c>
       <c r="D168" s="7" t="inlineStr">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="C169" s="6" t="inlineStr">
         <is>
-          <t>PLS. 3 LÜ EKO YEMEK SETİ BEYAZ</t>
+          <t>PLS. EKO YEMEK SETİ 3'lü BEYAZ</t>
         </is>
       </c>
       <c r="D169" s="8" t="inlineStr">
@@ -7542,7 +7542,7 @@
       </c>
       <c r="C172" s="6" t="inlineStr">
         <is>
-          <t>PLS. 2 Lİ PREMIUM YEMEK SETİ SİYAH</t>
+          <t>PLS. PREMIUM YEMEK SETİ 2'lü SİYAH</t>
         </is>
       </c>
       <c r="D172" s="7" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C173" s="6" t="inlineStr">
         <is>
-          <t>PLS. 3 LÜ EKO YEMEK SETİ BEYAZ</t>
+          <t>PLS. EKO YEMEK SETİ 3'lü BEYAZ</t>
         </is>
       </c>
       <c r="D173" s="8" t="inlineStr">
@@ -7829,7 +7829,7 @@
       </c>
       <c r="C179" s="6" t="inlineStr">
         <is>
-          <t>PLS. 4 LÜ PREMIUM YEMEK SETİ BEYAZ</t>
+          <t>PLS. PREMIUM YEMEK SETİ 4'lü BEYAZ</t>
         </is>
       </c>
       <c r="D179" s="8" t="inlineStr">
@@ -8649,7 +8649,7 @@
       </c>
       <c r="C199" s="6" t="inlineStr">
         <is>
-          <t>PLS. 3 LÜ PREMIUM YEMEK SETİ SİYAH</t>
+          <t>PLS. PREMIUM YEMEK SETİ 3'lü SİYAH</t>
         </is>
       </c>
       <c r="D199" s="8" t="inlineStr">
@@ -8977,7 +8977,7 @@
       </c>
       <c r="C207" s="6" t="inlineStr">
         <is>
-          <t>PLS. 4 LÜ EKO YEMEK SETİ BEYAZ</t>
+          <t>PLS. EKO YEMEK SETİ 4'lü BEYAZ</t>
         </is>
       </c>
       <c r="D207" s="8" t="inlineStr">
@@ -9223,7 +9223,7 @@
       </c>
       <c r="C213" s="6" t="inlineStr">
         <is>
-          <t>20'Lİ SHOT BARDAK 50 CC</t>
+          <t>SHOT BARDAK 50 CC</t>
         </is>
       </c>
       <c r="D213" s="8" t="inlineStr">
@@ -10166,7 +10166,7 @@
       </c>
       <c r="C236" s="6" t="inlineStr">
         <is>
-          <t>PLS. 5 Lİ EKO YEMEK SETİ BEYAZ</t>
+          <t>PLS. EKO YEMEK SETİ 5'lü BEYAZ</t>
         </is>
       </c>
       <c r="D236" s="7" t="inlineStr">
@@ -10863,7 +10863,7 @@
       </c>
       <c r="C253" s="6" t="inlineStr">
         <is>
-          <t>PLS. 2 Lİ PREMIUM YEMEK SETİ BEYAZ</t>
+          <t>PLS. PREMIUM YEMEK SETİ 2'lü BEYAZ</t>
         </is>
       </c>
       <c r="D253" s="8" t="inlineStr">
@@ -11150,7 +11150,7 @@
       </c>
       <c r="C260" s="6" t="inlineStr">
         <is>
-          <t>PLS. 5 Lİ PREMIUM YEMEK SETİ SİYAH</t>
+          <t>PLS. PREMIUM YEMEK SETİ 5'lü SİYAH</t>
         </is>
       </c>
       <c r="D260" s="7" t="inlineStr">
@@ -11396,7 +11396,7 @@
       </c>
       <c r="C266" s="6" t="inlineStr">
         <is>
-          <t>FERPROM PLS. PREMIUM SET (ÇATAL+ KAŞIK)</t>
+          <t>FERPROM PLS. PREMIUM SET 3'lü (ÇATAL+ KAŞIK)</t>
         </is>
       </c>
       <c r="D266" s="7" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="C278" s="6" t="inlineStr">
         <is>
-          <t>PLS. 6 LI PREMIUM YEMEK SETİ SİYAH</t>
+          <t>PLS. PREMIUM YEMEK SETİ 6'lü SİYAH</t>
         </is>
       </c>
       <c r="D278" s="7" t="inlineStr">
@@ -12175,7 +12175,7 @@
       </c>
       <c r="C285" s="6" t="inlineStr">
         <is>
-          <t>PLS. 2 Lİ EKO KAŞIK YEMEK SETİ ŞEFFAF</t>
+          <t>PLS. EKO KAŞIK YEMEK SETİ 2'lü ŞEFFAF</t>
         </is>
       </c>
       <c r="D285" s="8" t="inlineStr">
@@ -12913,7 +12913,7 @@
       </c>
       <c r="C303" s="6" t="inlineStr">
         <is>
-          <t>PLS. ELİTE 4 LÜ YEMEK SETİ SİYAH</t>
+          <t>PLS. ELİTE YEMEK SETİ 4'lü SİYAH</t>
         </is>
       </c>
       <c r="D303" s="8" t="inlineStr">
@@ -12954,7 +12954,7 @@
       </c>
       <c r="C304" s="6" t="inlineStr">
         <is>
-          <t>PLS. EKO KAŞIK 20 Lİ</t>
+          <t>PLS. EKO KAŞIK</t>
         </is>
       </c>
       <c r="D304" s="7" t="inlineStr">
@@ -13651,7 +13651,7 @@
       </c>
       <c r="C321" s="6" t="inlineStr">
         <is>
-          <t>PLS. EKO ÇATAL 20 Lİ</t>
+          <t>PLS. EKO ÇATAL</t>
         </is>
       </c>
       <c r="D321" s="8" t="inlineStr">
@@ -13938,7 +13938,7 @@
       </c>
       <c r="C328" s="6" t="inlineStr">
         <is>
-          <t>PLS. 4 LÜ PREMIUM YEMEK SETİ ŞEFFAF</t>
+          <t>PLS. PREMIUM YEMEK SETİ 4'lü ŞEFFAF</t>
         </is>
       </c>
       <c r="D328" s="7" t="inlineStr">
@@ -14840,7 +14840,7 @@
       </c>
       <c r="C350" s="6" t="inlineStr">
         <is>
-          <t>PLS. ELİTE 2 Lİ YEMEK SETİ BEYAZ</t>
+          <t>PLS. ELİTE YEMEK SETİ 2'lü BEYAZ</t>
         </is>
       </c>
       <c r="D350" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Taxonomy final: strip colors/prefixes from GenelUrunAdi, SET size preserved
</commit_message>
<xml_diff>
--- a/STOK_TAKSONOMT_DUZENLE.xlsx
+++ b/STOK_TAKSONOMT_DUZENLE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="STOK TAKSONOMİSİ" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="AÇIKLAMA" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STOK TAKSONOMİSİ" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AÇIKLAMA" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'STOK TAKSONOMİSİ'!$A$1:$I$466</definedName>
@@ -572,7 +572,7 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>PLS. DIAMOND ÇATAL</t>
+          <t>DIAMOND ÇATAL</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. PREMİUM ÇATAL</t>
+          <t>PREMİUM ÇATAL</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. EKO KAŞIK BEYAZ</t>
+          <t>EKO KAŞIK</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. EKO KAŞIK</t>
+          <t>EKO KAŞIK</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>PLS. DIAMOND BIÇAK</t>
+          <t>DIAMOND BIÇAK</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>PLS. DIAMOND KAŞIK</t>
+          <t>DIAMOND KAŞIK</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>AL BASSAM PLS. EKO KAŞIK BEYAZ</t>
+          <t>EKO KAŞIK</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. EKO ÇATAL BEYAZ</t>
+          <t>EKO ÇATAL</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK KAŞIK PREMİUM</t>
+          <t>KAŞIK PREMİUM</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -982,7 +982,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>COMFY PACK PREMIUM ÇATAL</t>
+          <t>PREMIUM ÇATAL</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>MYPAK (REUSABLE) PLASTİK ÇATAL SİYAH</t>
+          <t>ÇATAL</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>180 CC PLS. KRİSTAL BARDAK</t>
+          <t>180 CC KRİSTAL BARDAK</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. LÜX ÇATAL</t>
+          <t>LÜX ÇATAL</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>PLS. DIAMOND ÇATAL SİYAH</t>
+          <t>DIAMOND ÇATAL</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. EKO BIÇAK</t>
+          <t>EKO BIÇAK</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK ÇATAL ELİTE BEYAZ</t>
+          <t>ÇATAL ELİTE</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>ESTETIK PREMIUM FORK</t>
+          <t>PREMIUM FORK</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK HB-10 BEYAZ</t>
+          <t>TABAK HB-10</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PREMİUM ÇATAL ŞEFFAF</t>
+          <t>PREMİUM ÇATAL</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. LÜX BIÇAK</t>
+          <t>LÜX BIÇAK</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>PLS. DIAMOND YEMEK SETİ 4'lü ŞEFFAF</t>
+          <t>DIAMOND YEMEK SETİ 4'lü</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>ECO OTUS LUX FORK</t>
+          <t>LUX FORK</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK MB-3 SARI</t>
+          <t>TABAK MB-3</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK EKO ÇATAL BEYAZ</t>
+          <t>EKO ÇATAL</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. PREMİUM KAŞIK</t>
+          <t>PREMİUM KAŞIK</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>COMFY PACK PREMIUM KAŞIK</t>
+          <t>PREMIUM KAŞIK</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PREMİUM BIÇAK ŞEFFAF</t>
+          <t>PREMİUM BIÇAK</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>ESTETIK PREMIUM SPOON</t>
+          <t>PREMIUM SPOON</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK EKO KAŞIK BEYAZ</t>
+          <t>EKO KAŞIK</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. PREMİUM ÇATAL SİYAH</t>
+          <t>PREMİUM ÇATAL</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMİUM YEMEK SETİ 4'lü ŞEFFAF</t>
+          <t>PREMİUM YEMEK SETİ 4'lü</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>PLS. DIAMOND KAŞIK SİYAH</t>
+          <t>DIAMOND KAŞIK</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. PREMİUM BIÇAK</t>
+          <t>PREMİUM BIÇAK</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>DALGALI DONDURMA KAŞIK KIRMIZI</t>
+          <t>DALGALI DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK EKO SUP KAŞIK BEYAZ</t>
+          <t>EKO SUP KAŞIK</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK BIÇAK ELİTE BEYAZ</t>
+          <t>BIÇAK ELİTE</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
@@ -2417,7 +2417,7 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>AL BASSAM PLS. DIAMOND KAŞIK SİYAH</t>
+          <t>DIAMOND KAŞIK</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>PLS. DIAMOND BIÇAK SİYAH</t>
+          <t>DIAMOND BIÇAK</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
@@ -2540,7 +2540,7 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>PLS. EURO ÇATAL</t>
+          <t>EURO ÇATAL</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK MB-3 BEYAZ</t>
+          <t>TABAK MB-3</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>MYPAK (REUSABLE) PLASTİK ÇATAL ŞEFFAF</t>
+          <t>ÇATAL</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK KAŞIK ELİTE BEYAZ</t>
+          <t>KAŞIK ELİTE</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PREMİUM KAŞIK ŞEFFAF</t>
+          <t>PREMİUM KAŞIK</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>MYPAK (REUSABLE) PLASTİK KAŞIK SİYAH</t>
+          <t>KAŞIK</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK KRİSTAL BARDAK LÜX</t>
+          <t>KRİSTAL BARDAK LÜX</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>MYPAK (REUSABLE) PLASTİK KAŞIK ŞEFFAF</t>
+          <t>KAŞIK</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>DALGALI DONDURMA KAŞIK ŞEFFAF</t>
+          <t>DALGALI DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>PİZZA TRİPOT BEYAZ</t>
+          <t>PİZZA TRİPOT</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK MOD 2 BEYAZ</t>
+          <t>TABAK MOD 2</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. PREMİUM BIÇAK SİYAH</t>
+          <t>PREMİUM BIÇAK</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>PLS. SMART FORK TRANSPARENT</t>
+          <t>SMART FORK</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>PLS. KAHVE TIKACI SİYAH</t>
+          <t>KAHVE TIKACI</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>ECORE PLASTİK ÇATAL BEYAZ</t>
+          <t>ECORE ÇATAL</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK DIAMOND KAŞIK</t>
+          <t>DIAMOND KAŞIK</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
@@ -3319,7 +3319,7 @@
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. EKO BIÇAK BEYAZ</t>
+          <t>EKO BIÇAK</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK MOD 1 BEYAZ</t>
+          <t>TABAK MOD 1</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>PLS. DIAMOND YEMEK SETİ 3'lü</t>
+          <t>DIAMOND YEMEK SETİ 3'lü</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr">
@@ -3442,7 +3442,7 @@
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK MB-3 BEJ</t>
+          <t>TABAK MB-3 BEJ</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>Plastik Diamond Bıçak Şeffaf QP</t>
+          <t>Diamond Bıçak QP</t>
         </is>
       </c>
       <c r="D73" s="8" t="inlineStr">
@@ -3524,7 +3524,7 @@
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK ÇATAL LÜX BEYAZ</t>
+          <t>ÇATAL LÜX</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Plastik Diamond Çatal Şeffaf QP</t>
+          <t>Diamond Çatal QP</t>
         </is>
       </c>
       <c r="D75" s="8" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>PLS. DIAMOND YEMEK SETİ 4'lü BEYAZ</t>
+          <t>DIAMOND YEMEK SETİ 4'lü</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
@@ -3647,7 +3647,7 @@
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>PLS. DIAMOND YEMEK SETİ 3'lü SİYAH</t>
+          <t>DIAMOND YEMEK SETİ 3'lü</t>
         </is>
       </c>
       <c r="D77" s="8" t="inlineStr">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMİUM SET 4'lü SİYAH</t>
+          <t>PREMİUM SET 4'lü</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
@@ -3729,7 +3729,7 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMIUM YEMEK SETİ 6'lü</t>
+          <t>PREMIUM YEMEK SETİ 6'lü</t>
         </is>
       </c>
       <c r="D79" s="8" t="inlineStr">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK MOD 2 SİYAH</t>
+          <t>TABAK MOD 2</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
@@ -3852,7 +3852,7 @@
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. PREMİUM KAŞIK SİYAH</t>
+          <t>PREMİUM KAŞIK</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
@@ -3934,7 +3934,7 @@
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK EURO ÇATAL</t>
+          <t>EURO ÇATAL</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PREMİUM ÇATAL SİYAH</t>
+          <t>PREMİUM ÇATAL</t>
         </is>
       </c>
       <c r="D85" s="8" t="inlineStr">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMIUM YEMEK SETİ 4'lü BEYAZ</t>
+          <t>PREMIUM YEMEK SETİ 4'lü</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>FERPROM PLS. PREMIUM SET 3'lü (ÇATAL+ BIÇAK)</t>
+          <t>PREMIUM SET 3'lü (ÇATAL+ BIÇAK)</t>
         </is>
       </c>
       <c r="D87" s="8" t="inlineStr">
@@ -4098,7 +4098,7 @@
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>BEST PLS. YEMEK SET 3'lü ŞEFFAF</t>
+          <t>YEMEK SET 3'lü</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
@@ -4139,7 +4139,7 @@
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK DIAMOND ÇATAL</t>
+          <t>DIAMOND ÇATAL</t>
         </is>
       </c>
       <c r="D89" s="8" t="inlineStr">
@@ -4180,7 +4180,7 @@
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>2000 GR PLS. TABAK BEYAZ MOD 16-A</t>
+          <t>2000 GR TABAK MOD 16-A</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
@@ -4221,7 +4221,7 @@
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK HB-6 BEYAZ</t>
+          <t>TABAK HB-6</t>
         </is>
       </c>
       <c r="D91" s="8" t="inlineStr">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>PLS. ELİTE YEMEK SETİ 4'lü BEYAZ</t>
+          <t>ELİTE YEMEK SETİ 4'lü</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
@@ -4303,7 +4303,7 @@
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK 16-A BEYAZ</t>
+          <t>TABAK 16-A</t>
         </is>
       </c>
       <c r="D93" s="8" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>PLS. ELİTE YEMEK SETİ 3'lü BEYAZ</t>
+          <t>ELİTE YEMEK SETİ 3'lü</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. LÜX KAŞIK</t>
+          <t>LÜX KAŞIK</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
@@ -4549,7 +4549,7 @@
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK DIAMOND ÇATAL 1/1</t>
+          <t>DIAMOND ÇATAL 1/1</t>
         </is>
       </c>
       <c r="D99" s="8" t="inlineStr">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
-          <t>PLS. SMART FORK BLACK</t>
+          <t>SMART FORK</t>
         </is>
       </c>
       <c r="D101" s="8" t="inlineStr">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="C102" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK TABAK 500</t>
+          <t>TABAK 500</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
@@ -4754,7 +4754,7 @@
       </c>
       <c r="C104" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PREMIUM ÇATAL BEJ</t>
+          <t>PREMIUM ÇATAL BEJ</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
@@ -4795,7 +4795,7 @@
       </c>
       <c r="C105" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK MOD 1 SİYAH</t>
+          <t>TABAK MOD 1</t>
         </is>
       </c>
       <c r="D105" s="8" t="inlineStr">
@@ -4836,7 +4836,7 @@
       </c>
       <c r="C106" s="6" t="inlineStr">
         <is>
-          <t>PLS. EKO YEMEK SETİ 4'lü BEYAZ</t>
+          <t>EKO YEMEK SETİ 4'lü</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
@@ -4918,7 +4918,7 @@
       </c>
       <c r="C108" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK MB-2 BEYAZ</t>
+          <t>TABAK MB-2</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
@@ -5000,7 +5000,7 @@
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>BEST PLS. YEMEK SETi 4'lü ŞEFFAF</t>
+          <t>YEMEK SETi 4'lü</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
@@ -5041,7 +5041,7 @@
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. LÜX KAŞIK SİYAH</t>
+          <t>LÜX KAŞIK</t>
         </is>
       </c>
       <c r="D111" s="8" t="inlineStr">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="C113" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMIUM SET 3'lü SİYAH</t>
+          <t>PREMIUM SET 3'lü</t>
         </is>
       </c>
       <c r="D113" s="8" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C114" s="6" t="inlineStr">
         <is>
-          <t>PLS. DIAMOND ÇATAL SİYAH</t>
+          <t>DIAMOND ÇATAL</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
@@ -5205,7 +5205,7 @@
       </c>
       <c r="C115" s="6" t="inlineStr">
         <is>
-          <t>MYPAK(REUSABLE) PLASTİK BIÇAK SİYAH</t>
+          <t>(REUSABLE) BIÇAK</t>
         </is>
       </c>
       <c r="D115" s="8" t="inlineStr">
@@ -5246,7 +5246,7 @@
       </c>
       <c r="C116" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK KARIŞTIRICI ŞEFFAF</t>
+          <t>KARIŞTIRICI</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
@@ -5287,7 +5287,7 @@
       </c>
       <c r="C117" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK MB-2 SİYAH</t>
+          <t>TABAK MB-2</t>
         </is>
       </c>
       <c r="D117" s="8" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="C118" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK HB-6 BEYAZ</t>
+          <t>TABAK HB-6</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
@@ -5369,7 +5369,7 @@
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK 16-A SİYAH</t>
+          <t>TABAK 16-A</t>
         </is>
       </c>
       <c r="D119" s="8" t="inlineStr">
@@ -5410,7 +5410,7 @@
       </c>
       <c r="C120" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PREMİUM BIÇAK SİYAH</t>
+          <t>PREMİUM BIÇAK</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
@@ -5451,7 +5451,7 @@
       </c>
       <c r="C121" s="6" t="inlineStr">
         <is>
-          <t>1000 GR TABAK BEYAZ MOD 1</t>
+          <t>1000 GR TABAK MOD 1</t>
         </is>
       </c>
       <c r="D121" s="8" t="inlineStr">
@@ -5492,7 +5492,7 @@
       </c>
       <c r="C122" s="6" t="inlineStr">
         <is>
-          <t>PLS. 3.80 GR SMART ÇATAL SİYAH</t>
+          <t>3.80 GR SMART ÇATAL</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
@@ -5533,7 +5533,7 @@
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK HB-6 SARI</t>
+          <t>TABAK HB-6</t>
         </is>
       </c>
       <c r="D123" s="8" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="C124" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK HB-7 BEYAZ</t>
+          <t>TABAK HB-7</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
@@ -5615,7 +5615,7 @@
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMIUM YEMEK SETİ 3'lü BEYAZ</t>
+          <t>PREMIUM YEMEK SETİ 3'lü</t>
         </is>
       </c>
       <c r="D125" s="8" t="inlineStr">
@@ -5656,7 +5656,7 @@
       </c>
       <c r="C126" s="6" t="inlineStr">
         <is>
-          <t>PLS. DIAMOND YEMEK SETİ 3'lü BEYAZ</t>
+          <t>DIAMOND YEMEK SETİ 3'lü</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
@@ -5697,7 +5697,7 @@
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
-          <t>BEST PREMIUM ÇATAL ŞEFFAF</t>
+          <t>PREMIUM ÇATAL</t>
         </is>
       </c>
       <c r="D127" s="8" t="inlineStr">
@@ -5738,7 +5738,7 @@
       </c>
       <c r="C128" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PREMİUM ÇATAL BEYAZ</t>
+          <t>PREMİUM ÇATAL</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
@@ -5779,7 +5779,7 @@
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>COMFY PACK LÜKS CİPS ÇATALI RENKLİ</t>
+          <t>LÜKS CİPS ÇATALI</t>
         </is>
       </c>
       <c r="D129" s="8" t="inlineStr">
@@ -5902,7 +5902,7 @@
       </c>
       <c r="C132" s="6" t="inlineStr">
         <is>
-          <t>PLS. ÇATALLI KAŞIK TEKLİ PAKETTE</t>
+          <t>ÇATALLI KAŞIK TEKLİ PAKETTE</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
@@ -5943,7 +5943,7 @@
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK ÇATAL PLATINUM 1/1</t>
+          <t>ÇATAL PLATINUM 1/1</t>
         </is>
       </c>
       <c r="D133" s="8" t="inlineStr">
@@ -6025,7 +6025,7 @@
       </c>
       <c r="C135" s="6" t="inlineStr">
         <is>
-          <t>DALGALI DONDURMA KAŞIK ŞEFFAF 1/1</t>
+          <t>DALGALI DONDURMA KAŞIK 1/1</t>
         </is>
       </c>
       <c r="D135" s="8" t="inlineStr">
@@ -6066,7 +6066,7 @@
       </c>
       <c r="C136" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK EKO SUP KAŞIK BEYAZ</t>
+          <t>EKO SUP KAŞIK</t>
         </is>
       </c>
       <c r="D136" s="7" t="inlineStr">
@@ -6107,7 +6107,7 @@
       </c>
       <c r="C137" s="6" t="inlineStr">
         <is>
-          <t>1 BÖLMELİ PLASTİK TABAK</t>
+          <t>1 BÖLMELİ TABAK</t>
         </is>
       </c>
       <c r="D137" s="8" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="C138" s="6" t="inlineStr">
         <is>
-          <t>DALGALI DONDURMA KAŞIK SİYAH</t>
+          <t>DALGALI DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D138" s="7" t="inlineStr">
@@ -6189,7 +6189,7 @@
       </c>
       <c r="C139" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PREMİUM SUP KAŞIK</t>
+          <t>PREMİUM SUP KAŞIK</t>
         </is>
       </c>
       <c r="D139" s="8" t="inlineStr">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="C140" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. EKO ÇATAL</t>
+          <t>EKO ÇATAL</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
@@ -6271,7 +6271,7 @@
       </c>
       <c r="C141" s="6" t="inlineStr">
         <is>
-          <t>SET 6'lü SMARTPACK ŞEFFAF Ç+K</t>
+          <t>SET 6'lü Ç+K</t>
         </is>
       </c>
       <c r="D141" s="8" t="inlineStr">
@@ -6353,7 +6353,7 @@
       </c>
       <c r="C143" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK DIAMOND ÇATAL BEJ</t>
+          <t>DIAMOND ÇATAL BEJ</t>
         </is>
       </c>
       <c r="D143" s="8" t="inlineStr">
@@ -6435,7 +6435,7 @@
       </c>
       <c r="C145" s="6" t="inlineStr">
         <is>
-          <t>ECORE PLASTİK ÇATAL KIRMIZI</t>
+          <t>ECORE ÇATAL</t>
         </is>
       </c>
       <c r="D145" s="8" t="inlineStr">
@@ -6517,7 +6517,7 @@
       </c>
       <c r="C147" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK ÇATAL ELİTE BEYAZ</t>
+          <t>ÇATAL ELİTE</t>
         </is>
       </c>
       <c r="D147" s="8" t="inlineStr">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="C148" s="6" t="inlineStr">
         <is>
-          <t>EKOPRO ÇATAL BEYAZ</t>
+          <t>EKOPRO ÇATAL</t>
         </is>
       </c>
       <c r="D148" s="7" t="inlineStr">
@@ -6640,7 +6640,7 @@
       </c>
       <c r="C150" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK 27-C BEYAZ</t>
+          <t>TABAK 27-C</t>
         </is>
       </c>
       <c r="D150" s="7" t="inlineStr">
@@ -6681,7 +6681,7 @@
       </c>
       <c r="C151" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK 21MM</t>
+          <t>TABAK 21MM</t>
         </is>
       </c>
       <c r="D151" s="8" t="inlineStr">
@@ -6763,7 +6763,7 @@
       </c>
       <c r="C153" s="6" t="inlineStr">
         <is>
-          <t>500 GR TABAK SİYAH MOD 2</t>
+          <t>500 GR TABAK MOD 2</t>
         </is>
       </c>
       <c r="D153" s="8" t="inlineStr">
@@ -6804,7 +6804,7 @@
       </c>
       <c r="C154" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PREMİUM KAŞIK BEYAZ</t>
+          <t>PREMİUM KAŞIK</t>
         </is>
       </c>
       <c r="D154" s="7" t="inlineStr">
@@ -6845,7 +6845,7 @@
       </c>
       <c r="C155" s="6" t="inlineStr">
         <is>
-          <t>1000 GR TABAK SİYAH MOD 1</t>
+          <t>1000 GR TABAK MOD 1</t>
         </is>
       </c>
       <c r="D155" s="8" t="inlineStr">
@@ -6886,7 +6886,7 @@
       </c>
       <c r="C156" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK DIAMOND BIÇAK</t>
+          <t>DIAMOND BIÇAK</t>
         </is>
       </c>
       <c r="D156" s="7" t="inlineStr">
@@ -6927,7 +6927,7 @@
       </c>
       <c r="C157" s="6" t="inlineStr">
         <is>
-          <t>COMFY PACK PREMIUM BIÇAK</t>
+          <t>PREMIUM BIÇAK</t>
         </is>
       </c>
       <c r="D157" s="8" t="inlineStr">
@@ -6968,7 +6968,7 @@
       </c>
       <c r="C158" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK MOD 8-C BEYAZ</t>
+          <t>TABAK MOD 8-C</t>
         </is>
       </c>
       <c r="D158" s="7" t="inlineStr">
@@ -7050,7 +7050,7 @@
       </c>
       <c r="C160" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK ÇATAL PREMİUM</t>
+          <t>ÇATAL PREMİUM</t>
         </is>
       </c>
       <c r="D160" s="7" t="inlineStr">
@@ -7091,7 +7091,7 @@
       </c>
       <c r="C161" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK BIÇAK PREMİUM</t>
+          <t>BIÇAK PREMİUM</t>
         </is>
       </c>
       <c r="D161" s="8" t="inlineStr">
@@ -7132,7 +7132,7 @@
       </c>
       <c r="C162" s="6" t="inlineStr">
         <is>
-          <t>80x110 CM ENDÜSTRİYEL JUMBO BOY ÇÖP POŞETİ SİYAH 400 GR</t>
+          <t>80x110 CM ENDÜSTRİYEL JUMBO BOY ÇÖP POŞETİ 400 GR</t>
         </is>
       </c>
       <c r="D162" s="7" t="inlineStr">
@@ -7173,7 +7173,7 @@
       </c>
       <c r="C163" s="6" t="inlineStr">
         <is>
-          <t>CİPS ÇATALI RENKLİ (25*1000)</t>
+          <t>CİPS ÇATALI</t>
         </is>
       </c>
       <c r="D163" s="8" t="inlineStr">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C164" s="6" t="inlineStr">
         <is>
-          <t>FERPROM PLS. KRİSTAL BARDAK</t>
+          <t>KRİSTAL BARDAK</t>
         </is>
       </c>
       <c r="D164" s="7" t="inlineStr">
@@ -7296,7 +7296,7 @@
       </c>
       <c r="C166" s="6" t="inlineStr">
         <is>
-          <t>DALGALI DONDURMA KAŞIK BEYAZ</t>
+          <t>DALGALI DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D166" s="7" t="inlineStr">
@@ -7337,7 +7337,7 @@
       </c>
       <c r="C167" s="6" t="inlineStr">
         <is>
-          <t>500 GR TABAK BEYAZ MOD 2</t>
+          <t>500 GR TABAK MOD 2</t>
         </is>
       </c>
       <c r="D167" s="8" t="inlineStr">
@@ -7378,7 +7378,7 @@
       </c>
       <c r="C168" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMIUM YEMEK SETİ 3'lü BEYAZ</t>
+          <t>PREMIUM YEMEK SETİ 3'lü</t>
         </is>
       </c>
       <c r="D168" s="7" t="inlineStr">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="C169" s="6" t="inlineStr">
         <is>
-          <t>PLS. EKO YEMEK SETİ 3'lü BEYAZ</t>
+          <t>EKO YEMEK SETİ 3'lü</t>
         </is>
       </c>
       <c r="D169" s="8" t="inlineStr">
@@ -7460,7 +7460,7 @@
       </c>
       <c r="C170" s="6" t="inlineStr">
         <is>
-          <t>PLS TABAK  MB-1 SARI</t>
+          <t>PLS TABAK MB-1</t>
         </is>
       </c>
       <c r="D170" s="7" t="inlineStr">
@@ -7501,7 +7501,7 @@
       </c>
       <c r="C171" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK DONDURMA KAŞIK RENKLİ</t>
+          <t>DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D171" s="8" t="inlineStr">
@@ -7542,7 +7542,7 @@
       </c>
       <c r="C172" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMIUM YEMEK SETİ 2'lü SİYAH</t>
+          <t>PREMIUM YEMEK SETİ 2'lü</t>
         </is>
       </c>
       <c r="D172" s="7" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C173" s="6" t="inlineStr">
         <is>
-          <t>PLS. EKO YEMEK SETİ 3'lü BEYAZ</t>
+          <t>EKO YEMEK SETİ 3'lü</t>
         </is>
       </c>
       <c r="D173" s="8" t="inlineStr">
@@ -7624,7 +7624,7 @@
       </c>
       <c r="C174" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK EKO KAŞIK BEYAZ</t>
+          <t>EKO KAŞIK</t>
         </is>
       </c>
       <c r="D174" s="7" t="inlineStr">
@@ -7665,7 +7665,7 @@
       </c>
       <c r="C175" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PREMİUM SUP KAŞIK</t>
+          <t>PREMİUM SUP KAŞIK</t>
         </is>
       </c>
       <c r="D175" s="8" t="inlineStr">
@@ -7706,7 +7706,7 @@
       </c>
       <c r="C176" s="6" t="inlineStr">
         <is>
-          <t>AL BASSAM PLS. DIAMOND KAŞIK ŞEFFAF</t>
+          <t>DIAMOND KAŞIK</t>
         </is>
       </c>
       <c r="D176" s="7" t="inlineStr">
@@ -7747,7 +7747,7 @@
       </c>
       <c r="C177" s="6" t="inlineStr">
         <is>
-          <t>PLS. PLATINUM ÇATAL SİYAH</t>
+          <t>PLATINUM ÇATAL</t>
         </is>
       </c>
       <c r="D177" s="8" t="inlineStr">
@@ -7788,7 +7788,7 @@
       </c>
       <c r="C178" s="6" t="inlineStr">
         <is>
-          <t>95 MM DONDURMA KAŞIK ŞEFFAF</t>
+          <t>95 MM DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D178" s="7" t="inlineStr">
@@ -7829,7 +7829,7 @@
       </c>
       <c r="C179" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMIUM YEMEK SETİ 4'lü BEYAZ</t>
+          <t>PREMIUM YEMEK SETİ 4'lü</t>
         </is>
       </c>
       <c r="D179" s="8" t="inlineStr">
@@ -7870,7 +7870,7 @@
       </c>
       <c r="C180" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK ÇATAL PLATINUM SİYAH 1/1</t>
+          <t>ÇATAL PLATINUM 1/1</t>
         </is>
       </c>
       <c r="D180" s="7" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="C182" s="6" t="inlineStr">
         <is>
-          <t>DALGALI DONDURMA KAŞIK MAVİ</t>
+          <t>DALGALI DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D182" s="7" t="inlineStr">
@@ -7993,7 +7993,7 @@
       </c>
       <c r="C183" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK MB-1 BEYAZ</t>
+          <t>TABAK MB-1</t>
         </is>
       </c>
       <c r="D183" s="8" t="inlineStr">
@@ -8075,7 +8075,7 @@
       </c>
       <c r="C185" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK ÇATAL DIAMOND BEYAZ</t>
+          <t>ÇATAL DIAMOND</t>
         </is>
       </c>
       <c r="D185" s="8" t="inlineStr">
@@ -8116,7 +8116,7 @@
       </c>
       <c r="C186" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK EKO SUP KAŞIK ŞEFFAF</t>
+          <t>EKO SUP KAŞIK</t>
         </is>
       </c>
       <c r="D186" s="7" t="inlineStr">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="C187" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK DIAMOND KAŞIK 1/1</t>
+          <t>DIAMOND KAŞIK 1/1</t>
         </is>
       </c>
       <c r="D187" s="8" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="C188" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK EKO BIÇAK</t>
+          <t>EKO BIÇAK</t>
         </is>
       </c>
       <c r="D188" s="7" t="inlineStr">
@@ -8239,7 +8239,7 @@
       </c>
       <c r="C189" s="6" t="inlineStr">
         <is>
-          <t>PLS. VOTKA BARDAK</t>
+          <t>VOTKA BARDAK</t>
         </is>
       </c>
       <c r="D189" s="8" t="inlineStr">
@@ -8362,7 +8362,7 @@
       </c>
       <c r="C192" s="6" t="inlineStr">
         <is>
-          <t>2000 GR TABAK SİYAH MOD 16-A</t>
+          <t>2000 GR TABAK MOD 16-A</t>
         </is>
       </c>
       <c r="D192" s="7" t="inlineStr">
@@ -8403,7 +8403,7 @@
       </c>
       <c r="C193" s="6" t="inlineStr">
         <is>
-          <t>FAKTOR PLS. PREMIUM ÇATAL</t>
+          <t>FAKTOR PREMIUM ÇATAL</t>
         </is>
       </c>
       <c r="D193" s="8" t="inlineStr">
@@ -8444,7 +8444,7 @@
       </c>
       <c r="C194" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK EKO BIÇAK BEYAZ</t>
+          <t>EKO BIÇAK</t>
         </is>
       </c>
       <c r="D194" s="7" t="inlineStr">
@@ -8485,7 +8485,7 @@
       </c>
       <c r="C195" s="6" t="inlineStr">
         <is>
-          <t>ECORE PLASTİK TATLI KAŞIK BEYAZ</t>
+          <t>ECORE TATLI KAŞIK</t>
         </is>
       </c>
       <c r="D195" s="8" t="inlineStr">
@@ -8526,7 +8526,7 @@
       </c>
       <c r="C196" s="6" t="inlineStr">
         <is>
-          <t>SUP KAŞIK SİYAH</t>
+          <t>SUP KAŞIK</t>
         </is>
       </c>
       <c r="D196" s="7" t="inlineStr">
@@ -8567,7 +8567,7 @@
       </c>
       <c r="C197" s="6" t="inlineStr">
         <is>
-          <t>SUP KAŞIK ŞEFFAF</t>
+          <t>SUP KAŞIK</t>
         </is>
       </c>
       <c r="D197" s="8" t="inlineStr">
@@ -8608,7 +8608,7 @@
       </c>
       <c r="C198" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. LÜX BIÇAK SİYAH</t>
+          <t>LÜX BIÇAK</t>
         </is>
       </c>
       <c r="D198" s="7" t="inlineStr">
@@ -8649,7 +8649,7 @@
       </c>
       <c r="C199" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMIUM YEMEK SETİ 3'lü SİYAH</t>
+          <t>PREMIUM YEMEK SETİ 3'lü</t>
         </is>
       </c>
       <c r="D199" s="8" t="inlineStr">
@@ -8690,7 +8690,7 @@
       </c>
       <c r="C200" s="6" t="inlineStr">
         <is>
-          <t>2 BÖLMELİ PLASTİK TABAK</t>
+          <t>2 BÖLMELİ TABAK</t>
         </is>
       </c>
       <c r="D200" s="7" t="inlineStr">
@@ -8731,7 +8731,7 @@
       </c>
       <c r="C201" s="6" t="inlineStr">
         <is>
-          <t>PLS. ŞAMPANYA KADEHİ ŞEFFAF</t>
+          <t>ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D201" s="8" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="C202" s="6" t="inlineStr">
         <is>
-          <t>BIO ŞAMPANYA KADEHİ ŞEFFAF</t>
+          <t>ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D202" s="7" t="inlineStr">
@@ -8813,7 +8813,7 @@
       </c>
       <c r="C203" s="6" t="inlineStr">
         <is>
-          <t>PLS. PLATINUM ÇATAL</t>
+          <t>PLATINUM ÇATAL</t>
         </is>
       </c>
       <c r="D203" s="8" t="inlineStr">
@@ -8854,7 +8854,7 @@
       </c>
       <c r="C204" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK BIÇAK ELİTE BEYAZ</t>
+          <t>BIÇAK ELİTE</t>
         </is>
       </c>
       <c r="D204" s="7" t="inlineStr">
@@ -8895,7 +8895,7 @@
       </c>
       <c r="C205" s="6" t="inlineStr">
         <is>
-          <t>BIO PRIZMA KAP 200 CC</t>
+          <t>PRIZMA KAP 200 CC</t>
         </is>
       </c>
       <c r="D205" s="8" t="inlineStr">
@@ -8936,7 +8936,7 @@
       </c>
       <c r="C206" s="6" t="inlineStr">
         <is>
-          <t>PLS. MİNİ ŞARAP KADEHİ SİYAH</t>
+          <t>MİNİ ŞARAP KADEHİ</t>
         </is>
       </c>
       <c r="D206" s="7" t="inlineStr">
@@ -8977,7 +8977,7 @@
       </c>
       <c r="C207" s="6" t="inlineStr">
         <is>
-          <t>PLS. EKO YEMEK SETİ 4'lü BEYAZ</t>
+          <t>EKO YEMEK SETİ 4'lü</t>
         </is>
       </c>
       <c r="D207" s="8" t="inlineStr">
@@ -9018,7 +9018,7 @@
       </c>
       <c r="C208" s="6" t="inlineStr">
         <is>
-          <t>MYPAK (REUSABLE) PLASTİK KAŞIK BEYAZ</t>
+          <t>KAŞIK</t>
         </is>
       </c>
       <c r="D208" s="7" t="inlineStr">
@@ -9059,7 +9059,7 @@
       </c>
       <c r="C209" s="6" t="inlineStr">
         <is>
-          <t>BIO 200 cc  AYAKLI KASE</t>
+          <t>200 cc AYAKLI KASE</t>
         </is>
       </c>
       <c r="D209" s="8" t="inlineStr">
@@ -9141,7 +9141,7 @@
       </c>
       <c r="C211" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK MOD 7 BEYAZ</t>
+          <t>TABAK MOD 7</t>
         </is>
       </c>
       <c r="D211" s="8" t="inlineStr">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C214" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK DIAMOND BIÇAK BEJ</t>
+          <t>DIAMOND BIÇAK BEJ</t>
         </is>
       </c>
       <c r="D214" s="7" t="inlineStr">
@@ -9305,7 +9305,7 @@
       </c>
       <c r="C215" s="6" t="inlineStr">
         <is>
-          <t>AL BASSAM PLS. EKO ÇATAL SİYAH</t>
+          <t>EKO ÇATAL</t>
         </is>
       </c>
       <c r="D215" s="8" t="inlineStr">
@@ -9387,7 +9387,7 @@
       </c>
       <c r="C217" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK KARIŞTIRICI BEYAZ</t>
+          <t>KARIŞTIRICI</t>
         </is>
       </c>
       <c r="D217" s="8" t="inlineStr">
@@ -9510,7 +9510,7 @@
       </c>
       <c r="C220" s="6" t="inlineStr">
         <is>
-          <t>XPS HB-10 SANDVİÇ KABI BEYAZ</t>
+          <t>XPS HB-10 SANDVİÇ KABI</t>
         </is>
       </c>
       <c r="D220" s="7" t="inlineStr">
@@ -9551,7 +9551,7 @@
       </c>
       <c r="C221" s="6" t="inlineStr">
         <is>
-          <t>FAKTOR PLS. PREMIUM KAŞIK</t>
+          <t>FAKTOR PREMIUM KAŞIK</t>
         </is>
       </c>
       <c r="D221" s="8" t="inlineStr">
@@ -9592,7 +9592,7 @@
       </c>
       <c r="C222" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK BIÇAK PREMİUM BEYAZ</t>
+          <t>BIÇAK PREMİUM</t>
         </is>
       </c>
       <c r="D222" s="7" t="inlineStr">
@@ -9715,7 +9715,7 @@
       </c>
       <c r="C225" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK TABAK 27-B BEYAZ</t>
+          <t>TABAK 27-B</t>
         </is>
       </c>
       <c r="D225" s="8" t="inlineStr">
@@ -9756,7 +9756,7 @@
       </c>
       <c r="C226" s="6" t="inlineStr">
         <is>
-          <t>PS ECO KAŞIK BEYAZ 100*20</t>
+          <t>PS ECO KAŞIK</t>
         </is>
       </c>
       <c r="D226" s="7" t="inlineStr">
@@ -9838,7 +9838,7 @@
       </c>
       <c r="C228" s="6" t="inlineStr">
         <is>
-          <t>BIO SHOT BARDAK 40 CC</t>
+          <t>SHOT BARDAK 40 CC</t>
         </is>
       </c>
       <c r="D228" s="7" t="inlineStr">
@@ -9879,7 +9879,7 @@
       </c>
       <c r="C229" s="6" t="inlineStr">
         <is>
-          <t>MYPAK (REUSABLE) PLASTİK BIÇAK ŞEFFAF</t>
+          <t>BIÇAK</t>
         </is>
       </c>
       <c r="D229" s="8" t="inlineStr">
@@ -9920,7 +9920,7 @@
       </c>
       <c r="C230" s="6" t="inlineStr">
         <is>
-          <t>PLS. 3.80 GR SMART ÇATAL</t>
+          <t>3.80 GR SMART ÇATAL</t>
         </is>
       </c>
       <c r="D230" s="7" t="inlineStr">
@@ -9961,7 +9961,7 @@
       </c>
       <c r="C231" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK KAŞIK PREMİUM BEYAZ</t>
+          <t>KAŞIK PREMİUM</t>
         </is>
       </c>
       <c r="D231" s="8" t="inlineStr">
@@ -10043,7 +10043,7 @@
       </c>
       <c r="C233" s="6" t="inlineStr">
         <is>
-          <t>MYPAK (REUSABLE) PLASTİK BIÇAK BEYAZ</t>
+          <t>BIÇAK</t>
         </is>
       </c>
       <c r="D233" s="8" t="inlineStr">
@@ -10084,7 +10084,7 @@
       </c>
       <c r="C234" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. LÜX ÇATAL SİYAH</t>
+          <t>LÜX ÇATAL</t>
         </is>
       </c>
       <c r="D234" s="7" t="inlineStr">
@@ -10125,7 +10125,7 @@
       </c>
       <c r="C235" s="6" t="inlineStr">
         <is>
-          <t>LUSSO BIO PREMİUM ÇATAL</t>
+          <t>LUSSO PREMİUM ÇATAL</t>
         </is>
       </c>
       <c r="D235" s="8" t="inlineStr">
@@ -10166,7 +10166,7 @@
       </c>
       <c r="C236" s="6" t="inlineStr">
         <is>
-          <t>PLS. EKO YEMEK SETİ 5'lü BEYAZ</t>
+          <t>EKO YEMEK SETİ 5'lü</t>
         </is>
       </c>
       <c r="D236" s="7" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="C237" s="6" t="inlineStr">
         <is>
-          <t>BIO VİSKİ BARDAK 220 CC</t>
+          <t>VİSKİ BARDAK 220 CC</t>
         </is>
       </c>
       <c r="D237" s="8" t="inlineStr">
@@ -10248,7 +10248,7 @@
       </c>
       <c r="C238" s="6" t="inlineStr">
         <is>
-          <t>BIO PRİZMA KAP 120 CC</t>
+          <t>PRİZMA KAP 120 CC</t>
         </is>
       </c>
       <c r="D238" s="7" t="inlineStr">
@@ -10371,7 +10371,7 @@
       </c>
       <c r="C241" s="6" t="inlineStr">
         <is>
-          <t>COMFY PACK DIAMOND ÇATAL SİYAH</t>
+          <t>DIAMOND ÇATAL</t>
         </is>
       </c>
       <c r="D241" s="8" t="inlineStr">
@@ -10453,7 +10453,7 @@
       </c>
       <c r="C243" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PREMİUM KAŞIK SİYAH</t>
+          <t>PREMİUM KAŞIK</t>
         </is>
       </c>
       <c r="D243" s="8" t="inlineStr">
@@ -10494,7 +10494,7 @@
       </c>
       <c r="C244" s="6" t="inlineStr">
         <is>
-          <t>LUSSO BIO PREMİUM TATLI KAŞIK</t>
+          <t>LUSSO PREMİUM TATLI KAŞIK</t>
         </is>
       </c>
       <c r="D244" s="7" t="inlineStr">
@@ -10617,7 +10617,7 @@
       </c>
       <c r="C247" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK BIÇAK DIAMOND BEYAZ</t>
+          <t>BIÇAK DIAMOND</t>
         </is>
       </c>
       <c r="D247" s="8" t="inlineStr">
@@ -10658,7 +10658,7 @@
       </c>
       <c r="C248" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLASTİK ÇATAL LÜX</t>
+          <t>ÇATAL LÜX</t>
         </is>
       </c>
       <c r="D248" s="7" t="inlineStr">
@@ -10740,7 +10740,7 @@
       </c>
       <c r="C250" s="6" t="inlineStr">
         <is>
-          <t>LUSSO BIO PREMİUM KAŞIK</t>
+          <t>LUSSO PREMİUM KAŞIK</t>
         </is>
       </c>
       <c r="D250" s="7" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="C252" s="6" t="inlineStr">
         <is>
-          <t>ECORE PLASTİK KAŞIK BEYAZ</t>
+          <t>ECORE KAŞIK</t>
         </is>
       </c>
       <c r="D252" s="7" t="inlineStr">
@@ -10863,7 +10863,7 @@
       </c>
       <c r="C253" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMIUM YEMEK SETİ 2'lü BEYAZ</t>
+          <t>PREMIUM YEMEK SETİ 2'lü</t>
         </is>
       </c>
       <c r="D253" s="8" t="inlineStr">
@@ -10904,7 +10904,7 @@
       </c>
       <c r="C254" s="6" t="inlineStr">
         <is>
-          <t>1000 GR TABAK BEYAZ LÜX MOD 1</t>
+          <t>1000 GR TABAK LÜX MOD 1</t>
         </is>
       </c>
       <c r="D254" s="7" t="inlineStr">
@@ -10986,7 +10986,7 @@
       </c>
       <c r="C256" s="6" t="inlineStr">
         <is>
-          <t>2000 GR PLS. TABAK BEYAZ LÜX MOD 16-A</t>
+          <t>2000 GR TABAK LÜX MOD 16-A</t>
         </is>
       </c>
       <c r="D256" s="7" t="inlineStr">
@@ -11027,7 +11027,7 @@
       </c>
       <c r="C257" s="6" t="inlineStr">
         <is>
-          <t>PLS. tabak HB-10 BEYAZ</t>
+          <t>tabak HB-10</t>
         </is>
       </c>
       <c r="D257" s="8" t="inlineStr">
@@ -11068,7 +11068,7 @@
       </c>
       <c r="C258" s="6" t="inlineStr">
         <is>
-          <t>FAKTOR PLS. PREMIUM BIÇAK</t>
+          <t>FAKTOR PREMIUM BIÇAK</t>
         </is>
       </c>
       <c r="D258" s="7" t="inlineStr">
@@ -11109,7 +11109,7 @@
       </c>
       <c r="C259" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PANDA KAŞIK BEYAZ (16*500=8.000)</t>
+          <t>PANDA KAŞIK (16*500=8.000)</t>
         </is>
       </c>
       <c r="D259" s="8" t="inlineStr">
@@ -11150,7 +11150,7 @@
       </c>
       <c r="C260" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMIUM YEMEK SETİ 5'lü SİYAH</t>
+          <t>PREMIUM YEMEK SETİ 5'lü</t>
         </is>
       </c>
       <c r="D260" s="7" t="inlineStr">
@@ -11273,7 +11273,7 @@
       </c>
       <c r="C263" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK KAŞIK DIAMOND BEYAZ</t>
+          <t>KAŞIK DIAMOND</t>
         </is>
       </c>
       <c r="D263" s="8" t="inlineStr">
@@ -11314,7 +11314,7 @@
       </c>
       <c r="C264" s="6" t="inlineStr">
         <is>
-          <t>95 MM PLS. DONDURMA KAŞIK RENKLİ</t>
+          <t>95 MM DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D264" s="7" t="inlineStr">
@@ -11396,7 +11396,7 @@
       </c>
       <c r="C266" s="6" t="inlineStr">
         <is>
-          <t>FERPROM PLS. PREMIUM SET 3'lü (ÇATAL+ KAŞIK)</t>
+          <t>PREMIUM SET 3'lü (ÇATAL+ KAŞIK)</t>
         </is>
       </c>
       <c r="D266" s="7" t="inlineStr">
@@ -11437,7 +11437,7 @@
       </c>
       <c r="C267" s="6" t="inlineStr">
         <is>
-          <t>COMFY PACK DIAMOND BIÇAK SİYAH</t>
+          <t>DIAMOND BIÇAK</t>
         </is>
       </c>
       <c r="D267" s="8" t="inlineStr">
@@ -11478,7 +11478,7 @@
       </c>
       <c r="C268" s="6" t="inlineStr">
         <is>
-          <t>BIO ŞAMPANYA KADEHİ SİYAH</t>
+          <t>ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D268" s="7" t="inlineStr">
@@ -11519,7 +11519,7 @@
       </c>
       <c r="C269" s="6" t="inlineStr">
         <is>
-          <t>EKOPRO PLASTİK ÇATAL ŞEFFAF</t>
+          <t>EKOPRO ÇATAL</t>
         </is>
       </c>
       <c r="D269" s="8" t="inlineStr">
@@ -11560,7 +11560,7 @@
       </c>
       <c r="C270" s="6" t="inlineStr">
         <is>
-          <t>80x110 CM ENDÜSTRİYEL JUMBO BOY ÇÖP POŞETİ SİYAH 500 GR</t>
+          <t>80x110 CM ENDÜSTRİYEL JUMBO BOY ÇÖP POŞETİ 500 GR</t>
         </is>
       </c>
       <c r="D270" s="7" t="inlineStr">
@@ -11642,7 +11642,7 @@
       </c>
       <c r="C272" s="6" t="inlineStr">
         <is>
-          <t>XPS MB-1 BÖLMESİZ KAPAKLI KAP SİYAH</t>
+          <t>XPS MB-1 BÖLMESİZ KAPAKLI KAP</t>
         </is>
       </c>
       <c r="D272" s="7" t="inlineStr">
@@ -11683,7 +11683,7 @@
       </c>
       <c r="C273" s="6" t="inlineStr">
         <is>
-          <t>5 MM KAPRON SİYAH</t>
+          <t>5 MM KAPRON</t>
         </is>
       </c>
       <c r="D273" s="8" t="inlineStr">
@@ -11724,7 +11724,7 @@
       </c>
       <c r="C274" s="6" t="inlineStr">
         <is>
-          <t>BIO ŞAMPANYA KADEHİ TR. KIRMIZI</t>
+          <t>ŞAMPANYA KADEHİ TR.</t>
         </is>
       </c>
       <c r="D274" s="7" t="inlineStr">
@@ -11765,7 +11765,7 @@
       </c>
       <c r="C275" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PREMİUM BIÇAK BEYAZ</t>
+          <t>PREMİUM BIÇAK</t>
         </is>
       </c>
       <c r="D275" s="8" t="inlineStr">
@@ -11847,7 +11847,7 @@
       </c>
       <c r="C277" s="6" t="inlineStr">
         <is>
-          <t>PRİZMA KAP 200 CC SİYAH</t>
+          <t>PRİZMA KAP 200 CC</t>
         </is>
       </c>
       <c r="D277" s="8" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="C278" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMIUM YEMEK SETİ 6'lü SİYAH</t>
+          <t>PREMIUM YEMEK SETİ 6'lü</t>
         </is>
       </c>
       <c r="D278" s="7" t="inlineStr">
@@ -11929,7 +11929,7 @@
       </c>
       <c r="C279" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLASTİK KAŞIK LÜX</t>
+          <t>KAŞIK LÜX</t>
         </is>
       </c>
       <c r="D279" s="8" t="inlineStr">
@@ -11970,7 +11970,7 @@
       </c>
       <c r="C280" s="6" t="inlineStr">
         <is>
-          <t>BIO ŞAMPANYA KADEHİ GOLD</t>
+          <t>ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D280" s="7" t="inlineStr">
@@ -12052,7 +12052,7 @@
       </c>
       <c r="C282" s="6" t="inlineStr">
         <is>
-          <t>MYPAK (REUSABLE) PLASTİK ÇATAL BEYAZ</t>
+          <t>ÇATAL</t>
         </is>
       </c>
       <c r="D282" s="7" t="inlineStr">
@@ -12093,7 +12093,7 @@
       </c>
       <c r="C283" s="6" t="inlineStr">
         <is>
-          <t>ECORE PLASTİK BIÇAK BEYAZ</t>
+          <t>ECORE BIÇAK</t>
         </is>
       </c>
       <c r="D283" s="8" t="inlineStr">
@@ -12134,7 +12134,7 @@
       </c>
       <c r="C284" s="6" t="inlineStr">
         <is>
-          <t>BEST PREMIUM KAŞIK ŞEFFAF</t>
+          <t>PREMIUM KAŞIK</t>
         </is>
       </c>
       <c r="D284" s="7" t="inlineStr">
@@ -12175,7 +12175,7 @@
       </c>
       <c r="C285" s="6" t="inlineStr">
         <is>
-          <t>PLS. EKO KAŞIK YEMEK SETİ 2'lü ŞEFFAF</t>
+          <t>EKO KAŞIK YEMEK SETİ 2'lü</t>
         </is>
       </c>
       <c r="D285" s="8" t="inlineStr">
@@ -12257,7 +12257,7 @@
       </c>
       <c r="C287" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK BIÇAK ELİTE SİYAH</t>
+          <t>BIÇAK ELİTE</t>
         </is>
       </c>
       <c r="D287" s="8" t="inlineStr">
@@ -12298,7 +12298,7 @@
       </c>
       <c r="C288" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK KAŞIK PLATINUM SİYAH 1/1</t>
+          <t>KAŞIK PLATINUM 1/1</t>
         </is>
       </c>
       <c r="D288" s="7" t="inlineStr">
@@ -12339,7 +12339,7 @@
       </c>
       <c r="C289" s="6" t="inlineStr">
         <is>
-          <t>COMFY PACK DIAMOND KAŞIK SİYAH</t>
+          <t>DIAMOND KAŞIK</t>
         </is>
       </c>
       <c r="D289" s="8" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="C290" s="6" t="inlineStr">
         <is>
-          <t>BEST LUX BIÇAK ŞEFFAF</t>
+          <t>LUX BIÇAK</t>
         </is>
       </c>
       <c r="D290" s="7" t="inlineStr">
@@ -12544,7 +12544,7 @@
       </c>
       <c r="C294" s="6" t="inlineStr">
         <is>
-          <t>PLS. LÜX CİPS ÇATALI RENKLİ</t>
+          <t>LÜX CİPS ÇATALI</t>
         </is>
       </c>
       <c r="D294" s="7" t="inlineStr">
@@ -12585,7 +12585,7 @@
       </c>
       <c r="C295" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK EKO KAŞIK SİYAH</t>
+          <t>EKO KAŞIK</t>
         </is>
       </c>
       <c r="D295" s="8" t="inlineStr">
@@ -12626,7 +12626,7 @@
       </c>
       <c r="C296" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PANDA KAŞIK KIRMIZI (16*500=8.000)</t>
+          <t>PANDA KAŞIK (16*500=8.000)</t>
         </is>
       </c>
       <c r="D296" s="7" t="inlineStr">
@@ -12667,7 +12667,7 @@
       </c>
       <c r="C297" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK DIAMOND ÇATAL SİYAH</t>
+          <t>DIAMOND ÇATAL</t>
         </is>
       </c>
       <c r="D297" s="8" t="inlineStr">
@@ -12708,7 +12708,7 @@
       </c>
       <c r="C298" s="6" t="inlineStr">
         <is>
-          <t>CİPS ÇATALI KIRMIZI (25*1000)</t>
+          <t>CİPS ÇATALI</t>
         </is>
       </c>
       <c r="D298" s="7" t="inlineStr">
@@ -12749,7 +12749,7 @@
       </c>
       <c r="C299" s="6" t="inlineStr">
         <is>
-          <t>CİPS ÇATALI MAVİ (25*1000)</t>
+          <t>CİPS ÇATALI</t>
         </is>
       </c>
       <c r="D299" s="8" t="inlineStr">
@@ -12913,7 +12913,7 @@
       </c>
       <c r="C303" s="6" t="inlineStr">
         <is>
-          <t>PLS. ELİTE YEMEK SETİ 4'lü SİYAH</t>
+          <t>ELİTE YEMEK SETİ 4'lü</t>
         </is>
       </c>
       <c r="D303" s="8" t="inlineStr">
@@ -12954,7 +12954,7 @@
       </c>
       <c r="C304" s="6" t="inlineStr">
         <is>
-          <t>PLS. EKO KAŞIK</t>
+          <t>EKO KAŞIK</t>
         </is>
       </c>
       <c r="D304" s="7" t="inlineStr">
@@ -12995,7 +12995,7 @@
       </c>
       <c r="C305" s="6" t="inlineStr">
         <is>
-          <t>TOSA PREMİUM KAŞIK BEBE MAVİ</t>
+          <t>TOSA PREMİUM KAŞIK BEBE</t>
         </is>
       </c>
       <c r="D305" s="8" t="inlineStr">
@@ -13077,7 +13077,7 @@
       </c>
       <c r="C307" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK ÇATAL ELİTE SİYAH</t>
+          <t>ÇATAL ELİTE</t>
         </is>
       </c>
       <c r="D307" s="8" t="inlineStr">
@@ -13118,7 +13118,7 @@
       </c>
       <c r="C308" s="6" t="inlineStr">
         <is>
-          <t>TOSA PREMİUM KAŞIK YEŞİL</t>
+          <t>TOSA PREMİUM KAŞIK</t>
         </is>
       </c>
       <c r="D308" s="7" t="inlineStr">
@@ -13200,7 +13200,7 @@
       </c>
       <c r="C310" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK EKO KAŞIK SİYAH</t>
+          <t>EKO KAŞIK</t>
         </is>
       </c>
       <c r="D310" s="7" t="inlineStr">
@@ -13364,7 +13364,7 @@
       </c>
       <c r="C314" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK KAŞIK PLATINUM 1/1</t>
+          <t>KAŞIK PLATINUM 1/1</t>
         </is>
       </c>
       <c r="D314" s="7" t="inlineStr">
@@ -13405,7 +13405,7 @@
       </c>
       <c r="C315" s="6" t="inlineStr">
         <is>
-          <t>95 MM DONDURMA KAŞIK KIRMIZI</t>
+          <t>95 MM DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D315" s="8" t="inlineStr">
@@ -13446,7 +13446,7 @@
       </c>
       <c r="C316" s="6" t="inlineStr">
         <is>
-          <t>3 MM KAPRON BEYAZ</t>
+          <t>3 MM KAPRON</t>
         </is>
       </c>
       <c r="D316" s="7" t="inlineStr">
@@ -13528,7 +13528,7 @@
       </c>
       <c r="C318" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK KAŞIK ELİTE BEYAZ</t>
+          <t>KAŞIK ELİTE</t>
         </is>
       </c>
       <c r="D318" s="7" t="inlineStr">
@@ -13569,7 +13569,7 @@
       </c>
       <c r="C319" s="6" t="inlineStr">
         <is>
-          <t>90x120 CM 120 LT KONTEYNER ÇÖP POŞETİ SİYAH 600 GR</t>
+          <t>90x120 CM 120 LT KONTEYNER ÇÖP POŞETİ 600 GR</t>
         </is>
       </c>
       <c r="D319" s="8" t="inlineStr">
@@ -13651,7 +13651,7 @@
       </c>
       <c r="C321" s="6" t="inlineStr">
         <is>
-          <t>PLS. EKO ÇATAL</t>
+          <t>EKO ÇATAL</t>
         </is>
       </c>
       <c r="D321" s="8" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="C322" s="6" t="inlineStr">
         <is>
-          <t>PLS. TEKLİ PREMIUM TATLI KAŞIK SETİ BEYAZ</t>
+          <t>TEKLİ PREMIUM TATLI KAŞIK SETİ</t>
         </is>
       </c>
       <c r="D322" s="7" t="inlineStr">
@@ -13733,7 +13733,7 @@
       </c>
       <c r="C323" s="6" t="inlineStr">
         <is>
-          <t>PİZZA TRİPOT BEYAZ QP</t>
+          <t>PİZZA TRİPOT QP</t>
         </is>
       </c>
       <c r="D323" s="8" t="inlineStr">
@@ -13774,7 +13774,7 @@
       </c>
       <c r="C324" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK DIAMOND KAŞIK SİYAH</t>
+          <t>DIAMOND KAŞIK</t>
         </is>
       </c>
       <c r="D324" s="7" t="inlineStr">
@@ -13815,7 +13815,7 @@
       </c>
       <c r="C325" s="6" t="inlineStr">
         <is>
-          <t>65x80 CM END BÜYÜK BOY ÇÖP POŞETİ SİYAH 200 GR</t>
+          <t>65x80 CM END BÜYÜK BOY ÇÖP POŞETİ 200 GR</t>
         </is>
       </c>
       <c r="D325" s="8" t="inlineStr">
@@ -13856,7 +13856,7 @@
       </c>
       <c r="C326" s="6" t="inlineStr">
         <is>
-          <t>DERİN TABAK BEYAZ MOD 7</t>
+          <t>DERİN TABAK MOD 7</t>
         </is>
       </c>
       <c r="D326" s="7" t="inlineStr">
@@ -13938,7 +13938,7 @@
       </c>
       <c r="C328" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMIUM YEMEK SETİ 4'lü ŞEFFAF</t>
+          <t>PREMIUM YEMEK SETİ 4'lü</t>
         </is>
       </c>
       <c r="D328" s="7" t="inlineStr">
@@ -13979,7 +13979,7 @@
       </c>
       <c r="C329" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK KAŞIK LÜX BEYAZ</t>
+          <t>KAŞIK LÜX</t>
         </is>
       </c>
       <c r="D329" s="8" t="inlineStr">
@@ -14020,7 +14020,7 @@
       </c>
       <c r="C330" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK ÇATAL PREMİUM BEYAZ</t>
+          <t>ÇATAL PREMİUM</t>
         </is>
       </c>
       <c r="D330" s="7" t="inlineStr">
@@ -14061,7 +14061,7 @@
       </c>
       <c r="C331" s="6" t="inlineStr">
         <is>
-          <t>PLS. EKO ÇATAL ŞEFFAF</t>
+          <t>EKO ÇATAL</t>
         </is>
       </c>
       <c r="D331" s="8" t="inlineStr">
@@ -14102,7 +14102,7 @@
       </c>
       <c r="C332" s="6" t="inlineStr">
         <is>
-          <t>5 MM KAPRON BEYAZ</t>
+          <t>5 MM KAPRON</t>
         </is>
       </c>
       <c r="D332" s="7" t="inlineStr">
@@ -14143,7 +14143,7 @@
       </c>
       <c r="C333" s="6" t="inlineStr">
         <is>
-          <t>FERPROM EKO KAŞIK BEYAZ</t>
+          <t>EKO KAŞIK</t>
         </is>
       </c>
       <c r="D333" s="8" t="inlineStr">
@@ -14225,7 +14225,7 @@
       </c>
       <c r="C335" s="6" t="inlineStr">
         <is>
-          <t>95 MM DONDURMA KAŞIK SARI</t>
+          <t>95 MM DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D335" s="8" t="inlineStr">
@@ -14266,7 +14266,7 @@
       </c>
       <c r="C336" s="6" t="inlineStr">
         <is>
-          <t>95 MM DONDURMA KAŞIK SİYAH</t>
+          <t>95 MM DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D336" s="7" t="inlineStr">
@@ -14348,7 +14348,7 @@
       </c>
       <c r="C338" s="6" t="inlineStr">
         <is>
-          <t>BEST PLS. TATLI KAŞIK ŞEFFAF</t>
+          <t>TATLI KAŞIK</t>
         </is>
       </c>
       <c r="D338" s="7" t="inlineStr">
@@ -14389,7 +14389,7 @@
       </c>
       <c r="C339" s="6" t="inlineStr">
         <is>
-          <t>CİPS ÇATALI SİYAH (25*1000)</t>
+          <t>CİPS ÇATALI</t>
         </is>
       </c>
       <c r="D339" s="8" t="inlineStr">
@@ -14430,7 +14430,7 @@
       </c>
       <c r="C340" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK EKO ÇATAL SİYAH</t>
+          <t>EKO ÇATAL</t>
         </is>
       </c>
       <c r="D340" s="7" t="inlineStr">
@@ -14553,7 +14553,7 @@
       </c>
       <c r="C343" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK EKO ÇATAL BEYAZ</t>
+          <t>EKO ÇATAL</t>
         </is>
       </c>
       <c r="D343" s="8" t="inlineStr">
@@ -14594,7 +14594,7 @@
       </c>
       <c r="C344" s="6" t="inlineStr">
         <is>
-          <t>PLS. PREMIUM KAŞIK TEKLİ YEMEK SETİ</t>
+          <t>PREMIUM KAŞIK TEKLİ YEMEK SETİ</t>
         </is>
       </c>
       <c r="D344" s="7" t="inlineStr">
@@ -14635,7 +14635,7 @@
       </c>
       <c r="C345" s="6" t="inlineStr">
         <is>
-          <t>KILIÇ KÜRDAN RENKLİ (25*1000)</t>
+          <t>KILIÇ KÜRDAN</t>
         </is>
       </c>
       <c r="D345" s="8" t="inlineStr">
@@ -14676,7 +14676,7 @@
       </c>
       <c r="C346" s="6" t="inlineStr">
         <is>
-          <t>95 MM DONDURMA KAŞIK YEŞİL</t>
+          <t>95 MM DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D346" s="7" t="inlineStr">
@@ -14758,7 +14758,7 @@
       </c>
       <c r="C348" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK TABAK 120</t>
+          <t>TABAK 120</t>
         </is>
       </c>
       <c r="D348" s="7" t="inlineStr">
@@ -14799,7 +14799,7 @@
       </c>
       <c r="C349" s="6" t="inlineStr">
         <is>
-          <t>PLS.PREMIUM ÇATAL TEKLİ YEMEK SETİ</t>
+          <t>PREMIUM ÇATAL TEKLİ YEMEK SETİ</t>
         </is>
       </c>
       <c r="D349" s="8" t="inlineStr">
@@ -14840,7 +14840,7 @@
       </c>
       <c r="C350" s="6" t="inlineStr">
         <is>
-          <t>PLS. ELİTE YEMEK SETİ 2'lü BEYAZ</t>
+          <t>ELİTE YEMEK SETİ 2'lü</t>
         </is>
       </c>
       <c r="D350" s="7" t="inlineStr">
@@ -14963,7 +14963,7 @@
       </c>
       <c r="C353" s="6" t="inlineStr">
         <is>
-          <t>95 MM DONDURMA KAŞIK MAVİ</t>
+          <t>95 MM DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D353" s="8" t="inlineStr">
@@ -15045,7 +15045,7 @@
       </c>
       <c r="C355" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK DIAMOND KAŞIK BEJ</t>
+          <t>DIAMOND KAŞIK BEJ</t>
         </is>
       </c>
       <c r="D355" s="8" t="inlineStr">
@@ -15086,7 +15086,7 @@
       </c>
       <c r="C356" s="6" t="inlineStr">
         <is>
-          <t>FERPROM EKO ÇATAL BEYAZ</t>
+          <t>EKO ÇATAL</t>
         </is>
       </c>
       <c r="D356" s="7" t="inlineStr">
@@ -15168,7 +15168,7 @@
       </c>
       <c r="C358" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PREMIUM BIÇAK</t>
+          <t>PREMIUM BIÇAK</t>
         </is>
       </c>
       <c r="D358" s="7" t="inlineStr">
@@ -15250,7 +15250,7 @@
       </c>
       <c r="C360" s="6" t="inlineStr">
         <is>
-          <t>EKO SUP KAŞIK ŞEFFAF</t>
+          <t>EKO SUP KAŞIK</t>
         </is>
       </c>
       <c r="D360" s="7" t="inlineStr">
@@ -15332,7 +15332,7 @@
       </c>
       <c r="C362" s="6" t="inlineStr">
         <is>
-          <t>ELDİVEN NİTRİL SİYAH M</t>
+          <t>ELDİVEN NİTRİL M</t>
         </is>
       </c>
       <c r="D362" s="7" t="inlineStr">
@@ -15373,7 +15373,7 @@
       </c>
       <c r="C363" s="6" t="inlineStr">
         <is>
-          <t>ELDİVEN NİTRİL SİYAH L</t>
+          <t>ELDİVEN NİTRİL L</t>
         </is>
       </c>
       <c r="D363" s="8" t="inlineStr">
@@ -15414,7 +15414,7 @@
       </c>
       <c r="C364" s="6" t="inlineStr">
         <is>
-          <t>PLS. TUMBLER BARDAK 290 CC</t>
+          <t>TUMBLER BARDAK 290 CC</t>
         </is>
       </c>
       <c r="D364" s="7" t="inlineStr">
@@ -15455,7 +15455,7 @@
       </c>
       <c r="C365" s="6" t="inlineStr">
         <is>
-          <t>PLS. TEKLİ PREMIUM KAŞIK SETİ BEYAZ</t>
+          <t>TEKLİ PREMIUM KAŞIK SETİ</t>
         </is>
       </c>
       <c r="D365" s="8" t="inlineStr">
@@ -15496,7 +15496,7 @@
       </c>
       <c r="C366" s="6" t="inlineStr">
         <is>
-          <t>500 GR TABAK BEYAZ LÜX MOD 2</t>
+          <t>500 GR TABAK LÜX MOD 2</t>
         </is>
       </c>
       <c r="D366" s="7" t="inlineStr">
@@ -15578,7 +15578,7 @@
       </c>
       <c r="C368" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PREMİUM SUP KAŞIK SİYAH</t>
+          <t>PREMİUM SUP KAŞIK</t>
         </is>
       </c>
       <c r="D368" s="7" t="inlineStr">
@@ -15619,7 +15619,7 @@
       </c>
       <c r="C369" s="6" t="inlineStr">
         <is>
-          <t>DALGALI DONDURMA KAŞIK TURUNCU</t>
+          <t>DALGALI DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D369" s="8" t="inlineStr">
@@ -15660,7 +15660,7 @@
       </c>
       <c r="C370" s="6" t="inlineStr">
         <is>
-          <t>PLS. TABAK 17MM</t>
+          <t>TABAK 17MM</t>
         </is>
       </c>
       <c r="D370" s="7" t="inlineStr">
@@ -15701,7 +15701,7 @@
       </c>
       <c r="C371" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. PREMİUM ÇATAL GOLD</t>
+          <t>PREMİUM ÇATAL</t>
         </is>
       </c>
       <c r="D371" s="8" t="inlineStr">
@@ -15783,7 +15783,7 @@
       </c>
       <c r="C373" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. PREMİUM KAŞIK GOLD</t>
+          <t>PREMİUM KAŞIK</t>
         </is>
       </c>
       <c r="D373" s="8" t="inlineStr">
@@ -15824,7 +15824,7 @@
       </c>
       <c r="C374" s="6" t="inlineStr">
         <is>
-          <t>95 MM DONDURMA KAŞIK TURUNCU</t>
+          <t>95 MM DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D374" s="7" t="inlineStr">
@@ -15947,7 +15947,7 @@
       </c>
       <c r="C377" s="6" t="inlineStr">
         <is>
-          <t>PLS. PLATINUM KAŞIK SİYAH</t>
+          <t>PLATINUM KAŞIK</t>
         </is>
       </c>
       <c r="D377" s="8" t="inlineStr">
@@ -16111,7 +16111,7 @@
       </c>
       <c r="C381" s="6" t="inlineStr">
         <is>
-          <t>CİPS ÇATALI TURUNCU (25*1000)</t>
+          <t>CİPS ÇATALI</t>
         </is>
       </c>
       <c r="D381" s="8" t="inlineStr">
@@ -16152,7 +16152,7 @@
       </c>
       <c r="C382" s="6" t="inlineStr">
         <is>
-          <t>PLS. MİNİ ŞARAP KADEHİ ŞEFFAF</t>
+          <t>MİNİ ŞARAP KADEHİ</t>
         </is>
       </c>
       <c r="D382" s="7" t="inlineStr">
@@ -16193,7 +16193,7 @@
       </c>
       <c r="C383" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK EKO SUP KAŞIK SİYAH</t>
+          <t>EKO SUP KAŞIK</t>
         </is>
       </c>
       <c r="D383" s="8" t="inlineStr">
@@ -16234,7 +16234,7 @@
       </c>
       <c r="C384" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK EKO KAŞIK ŞEFFAF</t>
+          <t>EKO KAŞIK</t>
         </is>
       </c>
       <c r="D384" s="7" t="inlineStr">
@@ -16357,7 +16357,7 @@
       </c>
       <c r="C387" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK TABAK 250</t>
+          <t>TABAK 250</t>
         </is>
       </c>
       <c r="D387" s="8" t="inlineStr">
@@ -16398,7 +16398,7 @@
       </c>
       <c r="C388" s="6" t="inlineStr">
         <is>
-          <t>AL BASSAM PLS. EKO ÇATAL BEYAZ</t>
+          <t>EKO ÇATAL</t>
         </is>
       </c>
       <c r="D388" s="7" t="inlineStr">
@@ -16562,7 +16562,7 @@
       </c>
       <c r="C392" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK TABAK 750</t>
+          <t>TABAK 750</t>
         </is>
       </c>
       <c r="D392" s="7" t="inlineStr">
@@ -16685,7 +16685,7 @@
       </c>
       <c r="C395" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK TABAK 1500</t>
+          <t>TABAK 1500</t>
         </is>
       </c>
       <c r="D395" s="8" t="inlineStr">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="C397" s="6" t="inlineStr">
         <is>
-          <t>9 INC KRİSTAL PARTY TABAK SİYAH</t>
+          <t>9 INC KRİSTAL PARTY TABAK</t>
         </is>
       </c>
       <c r="D397" s="8" t="inlineStr">
@@ -16808,7 +16808,7 @@
       </c>
       <c r="C398" s="6" t="inlineStr">
         <is>
-          <t>9 INC KRİSTAL PARTY TABAK BEYAZ</t>
+          <t>9 INC KRİSTAL PARTY TABAK</t>
         </is>
       </c>
       <c r="D398" s="7" t="inlineStr">
@@ -16849,7 +16849,7 @@
       </c>
       <c r="C399" s="6" t="inlineStr">
         <is>
-          <t>DALGALI DONDURMA KAŞIK YEŞİL</t>
+          <t>DALGALI DONDURMA KAŞIK</t>
         </is>
       </c>
       <c r="D399" s="8" t="inlineStr">
@@ -16890,7 +16890,7 @@
       </c>
       <c r="C400" s="6" t="inlineStr">
         <is>
-          <t>FERPROM PLS. TEKLI PREMIUM KAŞIK SET</t>
+          <t>TEKLI PREMIUM KAŞIK SET</t>
         </is>
       </c>
       <c r="D400" s="7" t="inlineStr">
@@ -16931,7 +16931,7 @@
       </c>
       <c r="C401" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK EKO BIÇAK BEYAZ</t>
+          <t>EKO BIÇAK</t>
         </is>
       </c>
       <c r="D401" s="8" t="inlineStr">
@@ -17013,7 +17013,7 @@
       </c>
       <c r="C403" s="6" t="inlineStr">
         <is>
-          <t>FERPROM PLS. TEKLI PREMIUM ÇATAL SET</t>
+          <t>TEKLI PREMIUM ÇATAL SET</t>
         </is>
       </c>
       <c r="D403" s="8" t="inlineStr">
@@ -17054,7 +17054,7 @@
       </c>
       <c r="C404" s="6" t="inlineStr">
         <is>
-          <t>PİZZA TRİPOT KIRMIZI</t>
+          <t>PİZZA TRİPOT</t>
         </is>
       </c>
       <c r="D404" s="7" t="inlineStr">
@@ -17095,7 +17095,7 @@
       </c>
       <c r="C405" s="6" t="inlineStr">
         <is>
-          <t>PLS. ŞAMPANYA KADEHİ GOLD</t>
+          <t>ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D405" s="8" t="inlineStr">
@@ -17136,7 +17136,7 @@
       </c>
       <c r="C406" s="6" t="inlineStr">
         <is>
-          <t>PİZZA TRİPOT YEŞİL</t>
+          <t>PİZZA TRİPOT</t>
         </is>
       </c>
       <c r="D406" s="7" t="inlineStr">
@@ -17177,7 +17177,7 @@
       </c>
       <c r="C407" s="6" t="inlineStr">
         <is>
-          <t>UZUN KOKTEYL KARIŞTIRICI MİX KIRMIZI</t>
+          <t>UZUN KOKTEYL KARIŞTIRICI MİX</t>
         </is>
       </c>
       <c r="D407" s="8" t="inlineStr">
@@ -17259,7 +17259,7 @@
       </c>
       <c r="C409" s="6" t="inlineStr">
         <is>
-          <t>KISA KOKTEYL KARIŞTIRICI MİX KIRMIZI</t>
+          <t>KISA KOKTEYL KARIŞTIRICI MİX</t>
         </is>
       </c>
       <c r="D409" s="8" t="inlineStr">
@@ -17341,7 +17341,7 @@
       </c>
       <c r="C411" s="6" t="inlineStr">
         <is>
-          <t>KRİSTAL TABAK ŞEFFAF</t>
+          <t>KRİSTAL TABAK</t>
         </is>
       </c>
       <c r="D411" s="8" t="inlineStr">
@@ -17382,7 +17382,7 @@
       </c>
       <c r="C412" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK TABAK - 150</t>
+          <t>TABAK - 150</t>
         </is>
       </c>
       <c r="D412" s="7" t="inlineStr">
@@ -17423,7 +17423,7 @@
       </c>
       <c r="C413" s="6" t="inlineStr">
         <is>
-          <t>DERİN MANTAR KABI MAVİ MOD 7-M</t>
+          <t>DERİN MANTAR KABI MOD 7-M</t>
         </is>
       </c>
       <c r="D413" s="8" t="inlineStr">
@@ -17464,7 +17464,7 @@
       </c>
       <c r="C414" s="6" t="inlineStr">
         <is>
-          <t>ÇAY KAŞIĞI BEYAZ</t>
+          <t>ÇAY KAŞIĞI</t>
         </is>
       </c>
       <c r="D414" s="7" t="inlineStr">
@@ -17546,7 +17546,7 @@
       </c>
       <c r="C416" s="6" t="inlineStr">
         <is>
-          <t>UZUN KOKTEYL KARIŞTIRICI MİX MAVİ</t>
+          <t>UZUN KOKTEYL KARIŞTIRICI MİX</t>
         </is>
       </c>
       <c r="D416" s="7" t="inlineStr">
@@ -17587,7 +17587,7 @@
       </c>
       <c r="C417" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK PANDA KAŞIK TURUNCU (16*500=8.000)</t>
+          <t>PANDA KAŞIK (16*500=8.000)</t>
         </is>
       </c>
       <c r="D417" s="8" t="inlineStr">
@@ -17751,7 +17751,7 @@
       </c>
       <c r="C421" s="6" t="inlineStr">
         <is>
-          <t>PLS. MİNİ ÇATAL ŞEFFAF</t>
+          <t>MİNİ ÇATAL</t>
         </is>
       </c>
       <c r="D421" s="8" t="inlineStr">
@@ -17792,7 +17792,7 @@
       </c>
       <c r="C422" s="6" t="inlineStr">
         <is>
-          <t>PLS. MİNİ KAŞIK ŞEFFAF</t>
+          <t>MİNİ KAŞIK</t>
         </is>
       </c>
       <c r="D422" s="7" t="inlineStr">
@@ -17833,7 +17833,7 @@
       </c>
       <c r="C423" s="6" t="inlineStr">
         <is>
-          <t>FERPROM EKO BIÇAK BEYAZ</t>
+          <t>EKO BIÇAK</t>
         </is>
       </c>
       <c r="D423" s="8" t="inlineStr">
@@ -17874,7 +17874,7 @@
       </c>
       <c r="C424" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK KARIŞTIRICI</t>
+          <t>KARIŞTIRICI</t>
         </is>
       </c>
       <c r="D424" s="7" t="inlineStr">
@@ -17915,7 +17915,7 @@
       </c>
       <c r="C425" s="6" t="inlineStr">
         <is>
-          <t>SMARTPACK PLS. EKO BIÇAK SİYAH</t>
+          <t>EKO BIÇAK</t>
         </is>
       </c>
       <c r="D425" s="8" t="inlineStr">
@@ -17956,7 +17956,7 @@
       </c>
       <c r="C426" s="6" t="inlineStr">
         <is>
-          <t>7 INC ELEGANT TABAK BEYAZ</t>
+          <t>7 INC ELEGANT TABAK</t>
         </is>
       </c>
       <c r="D426" s="7" t="inlineStr">
@@ -17997,7 +17997,7 @@
       </c>
       <c r="C427" s="6" t="inlineStr">
         <is>
-          <t>7 INC ELEGANT TABAK SİYAH</t>
+          <t>7 INC ELEGANT TABAK</t>
         </is>
       </c>
       <c r="D427" s="8" t="inlineStr">
@@ -18079,7 +18079,7 @@
       </c>
       <c r="C429" s="6" t="inlineStr">
         <is>
-          <t>PLS. MİNİ ŞARAP KADEHİ TR. KIRMIZI</t>
+          <t>MİNİ ŞARAP KADEHİ TR.</t>
         </is>
       </c>
       <c r="D429" s="8" t="inlineStr">
@@ -18120,7 +18120,7 @@
       </c>
       <c r="C430" s="6" t="inlineStr">
         <is>
-          <t>PLS. ŞAMPANYA KADEHİ GÜMÜŞ</t>
+          <t>ŞAMPANYA KADEHİ</t>
         </is>
       </c>
       <c r="D430" s="7" t="inlineStr">
@@ -18161,7 +18161,7 @@
       </c>
       <c r="C431" s="6" t="inlineStr">
         <is>
-          <t>PLS. MİNİ ŞARAP KADEHİ GÜMÜŞ</t>
+          <t>MİNİ ŞARAP KADEHİ</t>
         </is>
       </c>
       <c r="D431" s="8" t="inlineStr">
@@ -18202,7 +18202,7 @@
       </c>
       <c r="C432" s="6" t="inlineStr">
         <is>
-          <t>PLS. MİNİ ŞARAP KADEHİ GOLD</t>
+          <t>MİNİ ŞARAP KADEHİ</t>
         </is>
       </c>
       <c r="D432" s="7" t="inlineStr">
@@ -18243,7 +18243,7 @@
       </c>
       <c r="C433" s="6" t="inlineStr">
         <is>
-          <t>PLS. ŞAMPANYA KADEHİ TR. KIRMIZI</t>
+          <t>ŞAMPANYA KADEHİ TR.</t>
         </is>
       </c>
       <c r="D433" s="8" t="inlineStr">
@@ -18284,7 +18284,7 @@
       </c>
       <c r="C434" s="6" t="inlineStr">
         <is>
-          <t>KISA KOKTEYL KARIŞTIRICI MİX MAVİ</t>
+          <t>KISA KOKTEYL KARIŞTIRICI MİX</t>
         </is>
       </c>
       <c r="D434" s="7" t="inlineStr">
@@ -18366,7 +18366,7 @@
       </c>
       <c r="C436" s="6" t="inlineStr">
         <is>
-          <t>KARE TABAK BEYAZ</t>
+          <t>KARE TABAK</t>
         </is>
       </c>
       <c r="D436" s="7" t="inlineStr">
@@ -18407,7 +18407,7 @@
       </c>
       <c r="C437" s="6" t="inlineStr">
         <is>
-          <t>KARE TABAK GOLD</t>
+          <t>KARE TABAK</t>
         </is>
       </c>
       <c r="D437" s="8" t="inlineStr">
@@ -18448,7 +18448,7 @@
       </c>
       <c r="C438" s="6" t="inlineStr">
         <is>
-          <t>KARE TABAK ŞEFFAF</t>
+          <t>KARE TABAK</t>
         </is>
       </c>
       <c r="D438" s="7" t="inlineStr">
@@ -18489,7 +18489,7 @@
       </c>
       <c r="C439" s="6" t="inlineStr">
         <is>
-          <t>KARE TABAK SİYAH</t>
+          <t>KARE TABAK</t>
         </is>
       </c>
       <c r="D439" s="8" t="inlineStr">
@@ -18530,7 +18530,7 @@
       </c>
       <c r="C440" s="6" t="inlineStr">
         <is>
-          <t>7 INC ÇORBA KASESİ SİYAH</t>
+          <t>7 INC ÇORBA KASESİ</t>
         </is>
       </c>
       <c r="D440" s="7" t="inlineStr">
@@ -18571,7 +18571,7 @@
       </c>
       <c r="C441" s="6" t="inlineStr">
         <is>
-          <t>7 INC ÇORBA KASESİ BEYAZ</t>
+          <t>7 INC ÇORBA KASESİ</t>
         </is>
       </c>
       <c r="D441" s="8" t="inlineStr">
@@ -18612,7 +18612,7 @@
       </c>
       <c r="C442" s="6" t="inlineStr">
         <is>
-          <t>7 INC ÇORBA KASESİ YEŞİL</t>
+          <t>7 INC ÇORBA KASESİ</t>
         </is>
       </c>
       <c r="D442" s="7" t="inlineStr">
@@ -18653,7 +18653,7 @@
       </c>
       <c r="C443" s="6" t="inlineStr">
         <is>
-          <t>7 INC ÇORBA KASESİ ŞEFFAF</t>
+          <t>7 INC ÇORBA KASESİ</t>
         </is>
       </c>
       <c r="D443" s="8" t="inlineStr">
@@ -18694,7 +18694,7 @@
       </c>
       <c r="C444" s="6" t="inlineStr">
         <is>
-          <t>5 INC SALATA KASESİ SİYAH</t>
+          <t>5 INC SALATA KASESİ</t>
         </is>
       </c>
       <c r="D444" s="7" t="inlineStr">
@@ -18735,7 +18735,7 @@
       </c>
       <c r="C445" s="6" t="inlineStr">
         <is>
-          <t>5 INC SALATA KASESİ ŞEFFAF</t>
+          <t>5 INC SALATA KASESİ</t>
         </is>
       </c>
       <c r="D445" s="8" t="inlineStr">
@@ -18776,7 +18776,7 @@
       </c>
       <c r="C446" s="6" t="inlineStr">
         <is>
-          <t>5 INC SALATA KASESİ BEYAZ</t>
+          <t>5 INC SALATA KASESİ</t>
         </is>
       </c>
       <c r="D446" s="7" t="inlineStr">
@@ -18817,7 +18817,7 @@
       </c>
       <c r="C447" s="6" t="inlineStr">
         <is>
-          <t>OVAL KASE ŞEFFAF</t>
+          <t>OVAL KASE</t>
         </is>
       </c>
       <c r="D447" s="8" t="inlineStr">
@@ -18858,7 +18858,7 @@
       </c>
       <c r="C448" s="6" t="inlineStr">
         <is>
-          <t>OVAL KASE BEYAZ</t>
+          <t>OVAL KASE</t>
         </is>
       </c>
       <c r="D448" s="7" t="inlineStr">
@@ -18899,7 +18899,7 @@
       </c>
       <c r="C449" s="6" t="inlineStr">
         <is>
-          <t>OVAL KASE SİYAH</t>
+          <t>OVAL KASE</t>
         </is>
       </c>
       <c r="D449" s="8" t="inlineStr">
@@ -18940,7 +18940,7 @@
       </c>
       <c r="C450" s="6" t="inlineStr">
         <is>
-          <t>KILIÇ KÜRDAN BEYAZ (25*1000)</t>
+          <t>KILIÇ KÜRDAN</t>
         </is>
       </c>
       <c r="D450" s="7" t="inlineStr">
@@ -18981,7 +18981,7 @@
       </c>
       <c r="C451" s="6" t="inlineStr">
         <is>
-          <t>KILIÇ KÜRDAN SİYAH (25*1000)</t>
+          <t>KILIÇ KÜRDAN</t>
         </is>
       </c>
       <c r="D451" s="8" t="inlineStr">
@@ -19022,7 +19022,7 @@
       </c>
       <c r="C452" s="6" t="inlineStr">
         <is>
-          <t>KILIÇ KÜRDAN MAVİ (25*1000)</t>
+          <t>KILIÇ KÜRDAN</t>
         </is>
       </c>
       <c r="D452" s="7" t="inlineStr">
@@ -19063,7 +19063,7 @@
       </c>
       <c r="C453" s="6" t="inlineStr">
         <is>
-          <t>KILIÇ KÜRDAN TURUNCU (25*1000)</t>
+          <t>KILIÇ KÜRDAN</t>
         </is>
       </c>
       <c r="D453" s="8" t="inlineStr">
@@ -19104,7 +19104,7 @@
       </c>
       <c r="C454" s="6" t="inlineStr">
         <is>
-          <t>KILIÇ KÜRDAN KIRMIZI (25*1000)</t>
+          <t>KILIÇ KÜRDAN</t>
         </is>
       </c>
       <c r="D454" s="7" t="inlineStr">
@@ -19145,7 +19145,7 @@
       </c>
       <c r="C455" s="6" t="inlineStr">
         <is>
-          <t>10 INC KRİSTAL PARTY TABAK BEYAZ</t>
+          <t>10 INC KRİSTAL PARTY TABAK</t>
         </is>
       </c>
       <c r="D455" s="8" t="inlineStr">
@@ -19186,7 +19186,7 @@
       </c>
       <c r="C456" s="6" t="inlineStr">
         <is>
-          <t>10 INC KRİSTAL PARTY TABAK ŞEFFAF</t>
+          <t>10 INC KRİSTAL PARTY TABAK</t>
         </is>
       </c>
       <c r="D456" s="7" t="inlineStr">
@@ -19227,7 +19227,7 @@
       </c>
       <c r="C457" s="6" t="inlineStr">
         <is>
-          <t>10 INC KRİSTAL PARTY TABAK SİYAH</t>
+          <t>10 INC KRİSTAL PARTY TABAK</t>
         </is>
       </c>
       <c r="D457" s="8" t="inlineStr">
@@ -19268,7 +19268,7 @@
       </c>
       <c r="C458" s="6" t="inlineStr">
         <is>
-          <t>10 INC KRİSTAL PARTY TABAK GOLD</t>
+          <t>10 INC KRİSTAL PARTY TABAK</t>
         </is>
       </c>
       <c r="D458" s="7" t="inlineStr">
@@ -19309,7 +19309,7 @@
       </c>
       <c r="C459" s="6" t="inlineStr">
         <is>
-          <t>UZUN KOKTEYL KARIŞTIRICI MİX YEŞİL</t>
+          <t>UZUN KOKTEYL KARIŞTIRICI MİX</t>
         </is>
       </c>
       <c r="D459" s="8" t="inlineStr">
@@ -19350,7 +19350,7 @@
       </c>
       <c r="C460" s="6" t="inlineStr">
         <is>
-          <t>9 INC ELEGANT TABAK BEYAZ</t>
+          <t>9 INC ELEGANT TABAK</t>
         </is>
       </c>
       <c r="D460" s="7" t="inlineStr">
@@ -19391,7 +19391,7 @@
       </c>
       <c r="C461" s="6" t="inlineStr">
         <is>
-          <t>9 INC ELEGANT TABAK SİYAH</t>
+          <t>9 INC ELEGANT TABAK</t>
         </is>
       </c>
       <c r="D461" s="8" t="inlineStr">
@@ -19432,7 +19432,7 @@
       </c>
       <c r="C462" s="6" t="inlineStr">
         <is>
-          <t>9 INC ELEGANT TABAK ŞEFFAF</t>
+          <t>9 INC ELEGANT TABAK</t>
         </is>
       </c>
       <c r="D462" s="7" t="inlineStr">
@@ -19473,7 +19473,7 @@
       </c>
       <c r="C463" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK TABAK 2000</t>
+          <t>TABAK 2000</t>
         </is>
       </c>
       <c r="D463" s="8" t="inlineStr">
@@ -19514,7 +19514,7 @@
       </c>
       <c r="C464" s="6" t="inlineStr">
         <is>
-          <t>PLASTİK BIÇAK PLATINUM SİYAH 1/1</t>
+          <t>BIÇAK PLATINUM 1/1</t>
         </is>
       </c>
       <c r="D464" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Reclassify MyPak reusable cutlery as Diamond series; rebuild data + Excel
</commit_message>
<xml_diff>
--- a/STOK_TAKSONOMT_DUZENLE.xlsx
+++ b/STOK_TAKSONOMT_DUZENLE.xlsx
@@ -628,7 +628,7 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Eko</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Eko</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Eko</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>ÇATAL</t>
+          <t>DIAMOND ÇATAL</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>MyPak</t>
+          <t>Diamond</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Eko</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -1448,7 +1448,7 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G35" s="8" t="inlineStr">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G39" s="8" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G43" s="8" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>ÇATAL</t>
+          <t>DIAMOND ÇATAL</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>MyPak</t>
+          <t>Diamond</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -2719,7 +2719,7 @@
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>KAŞIK</t>
+          <t>DIAMOND KAŞIK</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>MyPak</t>
+          <t>Diamond</t>
         </is>
       </c>
       <c r="G55" s="8" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t>Lux</t>
+          <t>Kristal</t>
         </is>
       </c>
       <c r="G57" s="8" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>KAŞIK</t>
+          <t>DIAMOND KAŞIK</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>MyPak</t>
+          <t>Diamond</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G63" s="8" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Eko</t>
         </is>
       </c>
       <c r="G69" s="8" t="inlineStr">
@@ -3703,7 +3703,7 @@
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="F82" s="7" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
@@ -3990,7 +3990,7 @@
       </c>
       <c r="F85" s="8" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G85" s="8" t="inlineStr">
@@ -5205,7 +5205,7 @@
       </c>
       <c r="C115" s="6" t="inlineStr">
         <is>
-          <t>(REUSABLE) BIÇAK</t>
+          <t>DIAMOND BIÇAK</t>
         </is>
       </c>
       <c r="D115" s="8" t="inlineStr">
@@ -5220,7 +5220,7 @@
       </c>
       <c r="F115" s="8" t="inlineStr">
         <is>
-          <t>MyPak</t>
+          <t>Diamond</t>
         </is>
       </c>
       <c r="G115" s="8" t="inlineStr">
@@ -5425,7 +5425,7 @@
       </c>
       <c r="F120" s="7" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G120" s="7" t="inlineStr">
@@ -5753,7 +5753,7 @@
       </c>
       <c r="F128" s="7" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G128" s="7" t="inlineStr">
@@ -6081,7 +6081,7 @@
       </c>
       <c r="F136" s="7" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Eko</t>
         </is>
       </c>
       <c r="G136" s="7" t="inlineStr">
@@ -6204,7 +6204,7 @@
       </c>
       <c r="F139" s="8" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G139" s="8" t="inlineStr">
@@ -6245,7 +6245,7 @@
       </c>
       <c r="F140" s="7" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Eko</t>
         </is>
       </c>
       <c r="G140" s="7" t="inlineStr">
@@ -6491,7 +6491,7 @@
       </c>
       <c r="F146" s="7" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G146" s="7" t="inlineStr">
@@ -6819,7 +6819,7 @@
       </c>
       <c r="F154" s="7" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G154" s="7" t="inlineStr">
@@ -7680,7 +7680,7 @@
       </c>
       <c r="F175" s="8" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G175" s="8" t="inlineStr">
@@ -8131,7 +8131,7 @@
       </c>
       <c r="F186" s="7" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Eko</t>
         </is>
       </c>
       <c r="G186" s="7" t="inlineStr">
@@ -9018,7 +9018,7 @@
       </c>
       <c r="C208" s="6" t="inlineStr">
         <is>
-          <t>KAŞIK</t>
+          <t>DIAMOND KAŞIK</t>
         </is>
       </c>
       <c r="D208" s="7" t="inlineStr">
@@ -9033,7 +9033,7 @@
       </c>
       <c r="F208" s="7" t="inlineStr">
         <is>
-          <t>MyPak</t>
+          <t>Diamond</t>
         </is>
       </c>
       <c r="G208" s="7" t="inlineStr">
@@ -9879,7 +9879,7 @@
       </c>
       <c r="C229" s="6" t="inlineStr">
         <is>
-          <t>BIÇAK</t>
+          <t>DIAMOND BIÇAK</t>
         </is>
       </c>
       <c r="D229" s="8" t="inlineStr">
@@ -9894,7 +9894,7 @@
       </c>
       <c r="F229" s="8" t="inlineStr">
         <is>
-          <t>MyPak</t>
+          <t>Diamond</t>
         </is>
       </c>
       <c r="G229" s="8" t="inlineStr">
@@ -10043,7 +10043,7 @@
       </c>
       <c r="C233" s="6" t="inlineStr">
         <is>
-          <t>BIÇAK</t>
+          <t>DIAMOND BIÇAK</t>
         </is>
       </c>
       <c r="D233" s="8" t="inlineStr">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="F233" s="8" t="inlineStr">
         <is>
-          <t>MyPak</t>
+          <t>Diamond</t>
         </is>
       </c>
       <c r="G233" s="8" t="inlineStr">
@@ -10125,7 +10125,7 @@
       </c>
       <c r="C235" s="6" t="inlineStr">
         <is>
-          <t>LUSSO PREMİUM ÇATAL</t>
+          <t>PREMİUM ÇATAL</t>
         </is>
       </c>
       <c r="D235" s="8" t="inlineStr">
@@ -10140,7 +10140,7 @@
       </c>
       <c r="F235" s="8" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G235" s="8" t="inlineStr">
@@ -10468,7 +10468,7 @@
       </c>
       <c r="F243" s="8" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G243" s="8" t="inlineStr">
@@ -10494,7 +10494,7 @@
       </c>
       <c r="C244" s="6" t="inlineStr">
         <is>
-          <t>LUSSO PREMİUM TATLI KAŞIK</t>
+          <t>PREMİUM TATLI KAŞIK</t>
         </is>
       </c>
       <c r="D244" s="7" t="inlineStr">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="F244" s="7" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G244" s="7" t="inlineStr">
@@ -10740,7 +10740,7 @@
       </c>
       <c r="C250" s="6" t="inlineStr">
         <is>
-          <t>LUSSO PREMİUM KAŞIK</t>
+          <t>PREMİUM KAŞIK</t>
         </is>
       </c>
       <c r="D250" s="7" t="inlineStr">
@@ -10755,7 +10755,7 @@
       </c>
       <c r="F250" s="7" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G250" s="7" t="inlineStr">
@@ -11780,7 +11780,7 @@
       </c>
       <c r="F275" s="8" t="inlineStr">
         <is>
-          <t>Standart</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G275" s="8" t="inlineStr">
@@ -12052,7 +12052,7 @@
       </c>
       <c r="C282" s="6" t="inlineStr">
         <is>
-          <t>ÇATAL</t>
+          <t>DIAMOND ÇATAL</t>
         </is>
       </c>
       <c r="D282" s="7" t="inlineStr">
@@ -12067,7 +12067,7 @@
       </c>
       <c r="F282" s="7" t="inlineStr">
         <is>
-          <t>MyPak</t>
+          <t>Diamond</t>
         </is>
       </c>
       <c r="G282" s="7" t="inlineStr">
@@ -15593,7 +15593,7 @@
       </c>
       <c r="F368" s="7" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G368" s="7" t="inlineStr">
@@ -15716,7 +15716,7 @@
       </c>
       <c r="F371" s="8" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G371" s="8" t="inlineStr">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="F373" s="8" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G373" s="8" t="inlineStr">
@@ -16208,7 +16208,7 @@
       </c>
       <c r="F383" s="8" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Eko</t>
         </is>
       </c>
       <c r="G383" s="8" t="inlineStr">
@@ -17930,7 +17930,7 @@
       </c>
       <c r="F425" s="8" t="inlineStr">
         <is>
-          <t>SmartPack</t>
+          <t>Eko</t>
         </is>
       </c>
       <c r="G425" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Remove emoji, uppercase product names, Eko→Eco dropdown, fix materials (MyPak=PS, Elite=PP)
</commit_message>
<xml_diff>
--- a/STOK_TAKSONOMT_DUZENLE.xlsx
+++ b/STOK_TAKSONOMT_DUZENLE.xlsx
@@ -1028,7 +1028,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>PP (Çok Kull.)</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>PP (Çok Kull.)</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
@@ -2668,7 +2668,7 @@
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>PP (Çok Kull.)</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>PP (Çok Kull.)</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
@@ -5210,7 +5210,7 @@
       </c>
       <c r="D115" s="8" t="inlineStr">
         <is>
-          <t>PP (Çok Kull.)</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="D147" s="8" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="E147" s="8" t="inlineStr">
@@ -8859,7 +8859,7 @@
       </c>
       <c r="D204" s="7" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="E204" s="7" t="inlineStr">
@@ -9023,7 +9023,7 @@
       </c>
       <c r="D208" s="7" t="inlineStr">
         <is>
-          <t>PP (Çok Kull.)</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="E208" s="7" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="D229" s="8" t="inlineStr">
         <is>
-          <t>PP (Çok Kull.)</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="E229" s="8" t="inlineStr">
@@ -10048,7 +10048,7 @@
       </c>
       <c r="D233" s="8" t="inlineStr">
         <is>
-          <t>PP (Çok Kull.)</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="E233" s="8" t="inlineStr">
@@ -12057,7 +12057,7 @@
       </c>
       <c r="D282" s="7" t="inlineStr">
         <is>
-          <t>PP (Çok Kull.)</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="E282" s="7" t="inlineStr">
@@ -12262,7 +12262,7 @@
       </c>
       <c r="D287" s="8" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="E287" s="8" t="inlineStr">
@@ -12918,7 +12918,7 @@
       </c>
       <c r="D303" s="8" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="E303" s="8" t="inlineStr">
@@ -13082,7 +13082,7 @@
       </c>
       <c r="D307" s="8" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="E307" s="8" t="inlineStr">
@@ -13533,7 +13533,7 @@
       </c>
       <c r="D318" s="7" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="E318" s="7" t="inlineStr">
@@ -14845,7 +14845,7 @@
       </c>
       <c r="D350" s="7" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="E350" s="7" t="inlineStr">

</xml_diff>